<commit_message>
Add Hanım/Bey hitap, web-verified leads (60/100), and batch merge tooling.
Expand verified_profile_fields via web research batch JSON and apply script; regenerate outreach outputs with hitap post-processing.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/outputs/linkedin_hr_growth_leads_100.xlsx
+++ b/outputs/linkedin_hr_growth_leads_100.xlsx
@@ -516,12 +516,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Üçay Mühendislik</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -532,7 +532,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -572,18 +572,18 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Merhaba Elif, HR alanındaki deneyiminizle çalışanların İngilizce yeterliliğini artırmanın önemini biliyorsunuz. Konuşarak Öğren ile, ekiplerinizi global işbirliklerine hazırlamak için online konuşma pratiği sunuyoruz. Detayları paylaşmak isterim.</t>
+          <t>Merhaba Elif Hanım, HR alanındaki deneyiminizle çalışanların İngilizce yeterliliğini artırmanın önemini biliyorsunuz. Konuşarak Öğren ile, ekiplerinizi global işbirliklerine hazırlamak için online konuşma pratiği sunuyoruz. Detayları paylaşmak isterim.</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
           <t>Konu: Ekiplerinizi Global İşbirliğine Hazırlayın
-Merhaba Elif,
+Merhaba Elif Hanım,
 HR profesyoneli olarak, ekip üyelerinizin İngilizce yeterliliklerinin ve global toplantılara katılım becerilerinin arttırılması gerektiğini biliyorum. Konuşarak Öğren, çalışanlarınıza online İngilizce konuşma pratiği sunarak, kendilerine olan güvenlerini artırmalarına ve uluslararası işbirliklerine daha etkili katılmalarına yardımcı olabilir.
 Detayları görüşmek isterseniz, sevinirim.
 Saygılarımla,
@@ -598,7 +598,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Merhaba Eylül, Antwell Suites İstanbul'da İnsan Kaynakları Müdürü olarak çalışan bir profesyonel olarak, ekiplerinizin global toplantılarda daha etkili iletişim kurabilmesi için İngilizce konuşma pratiğine ihtiyaç duyduğunuzu biliyorum. Bu konuda konuşmak ister misiniz?</t>
+          <t>Merhaba Eylül Hanım, Antwell Suites İstanbul'da İnsan Kaynakları Müdürü olarak çalışan bir profesyonel olarak, ekiplerinizin global toplantılarda daha etkili iletişim kurabilmesi için İngilizce konuşma pratiğine ihtiyaç duyduğunuzu biliyorum. Bu konuda konuşmak ister misiniz?</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -950,13 +950,13 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Merhaba Berkan, iletişim becerilerinin geliştirilmesi konusundaki çalışmalarınızı görüyorum. Kurumsal ekipler için İngilizce konuşma pratiği sağlıyor ve bu sayede global toplantılara hazırlığı artırıyoruz. Bir sohbet edelim mi?</t>
+          <t>Merhaba Berkan Bey, iletişim becerilerinin geliştirilmesi konusundaki çalışmalarınızı görüyorum. Kurumsal ekipler için İngilizce konuşma pratiği sağlıyor ve bu sayede global toplantılara hazırlığı artırıyoruz. Bir sohbet edelim mi?</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
           <t>Konu: Kurumsal Ekipler İçin İngilizce Konuşma Pratiği
-Merhaba Berkan,
+Merhaba Berkan Bey,
 Gelişen çalışanlarınızın İngilizce konuşma becerilerini artırmak ve global toplantılara hazırlıklarını güçlendirmek adına size yardımcı olabileceğimizi düşünüyorum. Konuşarak Öğren, kurumsal ekiplerin online İngilizce konuşma pratiği yapmasını sağlarken, gelişim takibi ve raporlama sunarak performanslarını artırmayı hedefliyor. İlgilenirseniz, sizinle bir görüşme ayarlamak isterim.
 Saygılarımla,
 [Adınız]
@@ -1044,13 +1044,13 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Merhaba Nihal, kurumunuzun global iş ilişkilerindeki iletişim becerilerini geliştirmeye yönelik çabalarınızı takdir ediyorum. Konuşarak Öğren olarak, çalışanlarınızın İngilizce konuşma pratiği yapmalarına yardımcı olabiliriz. Daha fazla bilgi almak ister misiniz?</t>
+          <t>Merhaba Nihal Hanım, kurumunuzun global iş ilişkilerindeki iletişim becerilerini geliştirmeye yönelik çabalarınızı takdir ediyorum. Konuşarak Öğren olarak, çalışanlarınızın İngilizce konuşma pratiği yapmalarına yardımcı olabiliriz. Daha fazla bilgi almak ister misiniz?</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
           <t>Konu: Çalışanlarınızın İletişim Becerilerini Geliştirin
-Merhaba Nihal,
+Merhaba Nihal Hanım,
 Naci Çorap San. ve Tic. A.Ş.'deki iletişim becerilerini güçlendirme çabalarınızı biliyorum. Global iş ortamında etkili iletişim, başarı için kritik öneme sahip. Biz, Konuşarak Öğren olarak, çalışanlarınıza online İngilizce konuşma pratiği sunarak, güvenli bir iletişim ortamı yaratmayı hedefliyoruz. Bu süreçte gelişimlerini takip edip raporlayarak, ihtiyaçlarınıza özel çözümler sunabiliriz. 
 Detayları konuşmak ister misiniz?
 Saygılarımla,
@@ -1137,13 +1137,13 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Merhaba Nursen, çalışanlarınızın İngilizce konuşma becerilerini geliştirmelerine yardımcı olabileceğimizi düşündüm. Kurumsal eğitim programlarımızla, global toplantılara hazırlıkları için pratik imkanı sunuyoruz. Görüşmek ister misiniz?</t>
+          <t>Merhaba Nursen Hanım, çalışanlarınızın İngilizce konuşma becerilerini geliştirmelerine yardımcı olabileceğimizi düşündüm. Kurumsal eğitim programlarımızla, global toplantılara hazırlıkları için pratik imkanı sunuyoruz. Görüşmek ister misiniz?</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
           <t>Konu: İngilizce Konuşma Becerilerini Geliştirme Fırsatı
-Merhaba Nursen,
+Merhaba Nursen Hanım,
 Sektör Kimya'daki çalışanlarınızın İngilizce konuşma becerilerindeki eksiklikleri gidermeye yardımcı olabileceğimizi düşünüyorum. Kurumsal eğitim programlarımızla, global toplantılara daha iyi hazırlanmalarına ve iletişim becerilerini geliştirmelerine destek sunuyoruz. 
 Daha fazla bilgi almak isterseniz, sizinle görüşmek isterim.
 İyi çalışmalar,
@@ -1230,7 +1230,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Merhaba Sevda, global etkileşimlerde iletişim becerilerinin önemi gün geçtikçe artıyor. Konuşarak Öğren ile ekibinizin İngilizce konuşma pratiğini geliştirerek bu süreci destekleyebiliriz. Detayları paylaşmak isterim. Selamlar!</t>
+          <t>Merhaba Sevda Hanım, global etkileşimlerde iletişim becerilerinin önemi gün geçtikçe artıyor. Konuşarak Öğren ile ekibinizin İngilizce konuşma pratiğini geliştirerek bu süreci destekleyebiliriz. Detayları paylaşmak isterim. Selamlar!</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -1323,13 +1323,13 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Merhaba Burak, global iş ortamında ekiplerin İngilizce konuşma becerilerini artırmak için neler yapıyorsunuz? Konuşarak Öğren ile kurumsal ekiplerinize online pratik imkanı sunarak özgüven kazandırmayı hedefliyoruz. Detayları paylaşmak isterim.</t>
+          <t>Merhaba Burak Bey, global iş ortamında ekiplerin İngilizce konuşma becerilerini artırmak için neler yapıyorsunuz? Konuşarak Öğren ile kurumsal ekiplerinize online pratik imkanı sunarak özgüven kazandırmayı hedefliyoruz. Detayları paylaşmak isterim.</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
           <t>Konu: Ekiplerinizin İngilizce Konuşma Becerilerini Geliştirin
-Merhaba Burak,
+Merhaba Burak Bey,
 Gelişen global iş ortamında, ekiplerinizin İngilizce konuşma becerilerini artırmak kritik bir öneme sahip. Konuşarak Öğren, kurumsal ekiplerinize online İngilizce konuşma pratiği sunarak, özgüven kazanmalarına yardımcı oluyor. 
 Hedefimiz, HR profesyonellerinin global toplantılarda etkili iletişim kurma ihtiyaçlarına yanıt vermek. Eğer bu konuda daha fazla bilgi almak isterseniz, sizinle görüşmekten mutluluk duyarım.
 İyi çalışmalar,
@@ -1416,13 +1416,13 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Merhaba Şefaat Bey, Kırar Holding'deki insan kaynakları süreçlerinizi takip ediyorum. Kurumsal ekipler için İngilizce konuşma pratiği ve gelişim takibi sunuyoruz. Global pazarlarda iletişim yetkinliğini artırmanın yollarını keşfetmek ister misiniz?</t>
+          <t>Merhaba Şefaat Hanım, Kırar Holding'deki insan kaynakları süreçlerinizi takip ediyorum. Kurumsal ekipler için İngilizce konuşma pratiği ve gelişim takibi sunuyoruz. Global pazarlarda iletişim yetkinliğini artırmanın yollarını keşfetmek ister misiniz?</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
           <t>Konu: Ekiplerinizin İngilizce Konuşma Yetkinliğini Artırın
-Merhaba Şefaat Bey,
+Merhaba Şefaat Hanım,
 Kırar Holding'deki ekiplerinizin global pazarlarda etkili iletişim kurabilmesi için İngilizce konuşma pratiği sunuyoruz. Online platformumuz, çalışanlarınızın konuşma güvenini artırırken, gelişim takibi ve raporlama imkanı da sağlıyor. Global toplantılara daha iyi hazırlanmaları için nasıl destek olabileceğimizi konuşmak ister misiniz?
 İyi çalışmalar,
 [Adınız]
@@ -1509,7 +1509,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Merhaba Esra, Bilek İstanbul'da çalışanların global iletişim becerilerini geliştirmek için bir çözüm arayışında olduğunuzu anlıyorum. Konuşarak Öğren, ekiplerinizi online İngilizce konuşma pratiği ile güçlendirmeye yardımcı olabilir. Görüşmek ister misiniz?</t>
+          <t>Merhaba Esra Hanım, Bilek İstanbul'da çalışanların global iletişim becerilerini geliştirmek için bir çözüm arayışında olduğunuzu anlıyorum. Konuşarak Öğren, ekiplerinizi online İngilizce konuşma pratiği ile güçlendirmeye yardımcı olabilir. Görüşmek ister misiniz?</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Adil Işık Group</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1598,12 +1598,12 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>100</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Merhaba Pervin, İngilizce iletişimde güven artırma konusunda çalışan bir HR profesyoneli olarak, ekibinizin uluslararası toplantılarda daha hazır olmasına yardımcı olabileceğimi düşünüyorum. Konuşarak Öğren ile detayları paylaşmak isterim. Görüşmek üzere!</t>
+          <t>Merhaba Pervin Hanım, İngilizce iletişimde güven artırma konusunda çalışan bir HR profesyoneli olarak, ekibinizin uluslararası toplantılarda daha hazır olmasına yardımcı olabileceğimi düşünüyorum. Konuşarak Öğren ile detayları paylaşmak isterim. Görüşmek üzere!</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -1622,7 +1622,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -1695,7 +1695,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Merhaba Merve, İngilizce konuşma pratiği ve gelişim takibi konusunda destek sunuyoruz. Çalışanlarınızın kendine güvenini artırmalarına ve global toplantılara hazır olmalarına yardımcı olabileceğimizi düşünüyorum. Tanışmak ister misiniz?</t>
+          <t>Merhaba Merve Hanım, İngilizce konuşma pratiği ve gelişim takibi konusunda destek sunuyoruz. Çalışanlarınızın kendine güvenini artırmalarına ve global toplantılara hazır olmalarına yardımcı olabileceğimizi düşünüyorum. Tanışmak ister misiniz?</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -1975,7 +1975,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Merhaba Ceren, çalışanlarınızın İngilizce konuşma becerilerini geliştirmek, iletişim ve küresel işbirliği konularında yaşadıkları zorlukları aşmalarına yardımcı olabileceğimize inanıyorum. Konuşarak Öğren ile bu konuda nasıl destek olabileceğimizi konuşmak ister misiniz?</t>
+          <t>Merhaba Ceren Hanım, çalışanlarınızın İngilizce konuşma becerilerini geliştirmek, iletişim ve küresel işbirliği konularında yaşadıkları zorlukları aşmalarına yardımcı olabileceğimize inanıyorum. Konuşarak Öğren ile bu konuda nasıl destek olabileceğimizi konuşmak ister misiniz?</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -2068,13 +2068,13 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Merhaba Tuğçe, global toplantılardaki iletişim zorluklarını aşmak için ekibinize online İngilizce konuşma pratiği sunuyoruz. İletişim becerilerini geliştirmek ve toplantılara daha hazır girmek için nasıl yardımcı olabileceğimizi konuşmak ister misiniz?</t>
+          <t>Merhaba Tuğçe Hanım, global toplantılardaki iletişim zorluklarını aşmak için ekibinize online İngilizce konuşma pratiği sunuyoruz. İletişim becerilerini geliştirmek ve toplantılara daha hazır girmek için nasıl yardımcı olabileceğimizi konuşmak ister misiniz?</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
           <t>Konu: Ekibinizin İletişim Becerilerini Geliştirin
-Merhaba Tuğçe,
+Merhaba Tuğçe Hanım,
 Kurumsal ekiplere yönelik sunduğumuz online İngilizce konuşma pratiği, gelişim takibi ve raporlama hizmeti ile global toplantılardaki iletişim zorluklarını aşmanıza yardımcı olabiliriz. Ekibinizin kendine güvenini artırarak, etkili iletişim kurmalarını sağlamak istiyoruz. Bu konuda nasıl bir yol alabileceğimiz hakkında bir görüşme ayarlamak ister misiniz?
 İlginiz için teşekkürler,
 [Adınız]  
@@ -2100,12 +2100,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Uçak Tekstil</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2116,7 +2116,7 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Aydın, Turkey</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2156,18 +2156,18 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>95</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Merhaba Latife, HR profesyonellerinin dil becerilerini geliştirmeye yönelik çalışmalarda oldukça etkili olabileceğini düşünüyorum. Konuşarak Öğren ile ekip üyelerinizin İngilizce konuşma güvenini artırarak global iletişimde daha etkili olmalarına yardımcı olabiliriz. Görüşmek ister misiniz?</t>
+          <t>Merhaba Latife Hanım, HR profesyonellerinin dil becerilerini geliştirmeye yönelik çalışmalarda oldukça etkili olabileceğini düşünüyorum. Konuşarak Öğren ile ekip üyelerinizin İngilizce konuşma güvenini artırarak global iletişimde daha etkili olmalarına yardımcı olabiliriz. Görüşmek ister misiniz?</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
           <t>Konu: Ekip İletişimini Güçlendirin
-Merhaba Latife,
+Merhaba Latife Hanım,
 Kurumsal ekibinizin global toplantılarda daha güçlü bir iletişim kurmasını sağlamak için İngilizce konuşma pratiği sunuyoruz. Konuşarak Öğren ile çalışanlarınızın konuşma güvenini artırarak, çeşitli takımlarda etkili bir iletişim sağlamalarına yardımcı olabiliriz. Bu konuda bir görüşme yapmak ister misiniz?
 Sevgiler,
 [Adınız]
@@ -2181,7 +2181,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -2346,13 +2346,13 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Merhaba Ümmühan, iletişim becerilerinin global iş dünyasında ne kadar önemli olduğunu biliyoruz. Konuşarak Öğren ile ekibinizin İngilizce konuşma becerilerini geliştirmesine yardımcı olabiliriz. Detayları konuşmak ister misiniz?</t>
+          <t>Merhaba Ümmühan Bey, iletişim becerilerinin global iş dünyasında ne kadar önemli olduğunu biliyoruz. Konuşarak Öğren ile ekibinizin İngilizce konuşma becerilerini geliştirmesine yardımcı olabiliriz. Detayları konuşmak ister misiniz?</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
           <t>Konu: Ekibinizin İletişim Becerilerini Geliştirin
-Merhaba Ümmühan,
+Merhaba Ümmühan Bey,
 Global iş dünyasında etkili iletişim, başarıyı belirleyen kritik bir faktördür. Konuşarak Öğren olarak, kurumsal ekiplerinize online İngilizce konuşma pratiği sunarak, çalışanlarınızın özgüvenini artırmayı ve global toplantılara hazırlıklarını geliştirmeyi hedefliyoruz. İş birliğimiz sayesinde, ekibinizin performansını önemli ölçüde artırabiliriz. Detayları görüşmek için uygun bir zamanınız var mı?
 İyi çalışmalar dilerim,
 [Adınız]  
@@ -2379,12 +2379,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Süvari</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>Grup İnsan Kaynakları ve İdari İşler Müdürü</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2395,7 +2395,7 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2435,18 +2435,18 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>95</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Merhaba Nazan, kurumsal ekiplerdeki İngilizce konuşma pratiği ile ilgili zorlukları bildiğinizi düşünüyorum. Konuşarak Öğren olarak, ekiplerinizi global toplantılara daha iyi hazırlamak için online çözümler sunuyoruz. Detayları konuşmak ister misiniz?</t>
+          <t>Merhaba Nazan Hanım, kurumsal ekiplerdeki İngilizce konuşma pratiği ile ilgili zorlukları bildiğinizi düşünüyorum. Konuşarak Öğren olarak, ekiplerinizi global toplantılara daha iyi hazırlamak için online çözümler sunuyoruz. Detayları konuşmak ister misiniz?</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
           <t>Konu: Ekipleriniz İçin İngilizce Konuşma Pratiği
-Merhaba Nazan,
+Merhaba Nazan Hanım,
 Şirketinizin global toplantılarda daha fazla başarı elde etmesi için ekiplerinizin İngilizce konuşma becerilerini geliştirmek önem taşıyor. Konuşarak Öğren olarak, kurumsal ekipler için online İngilizce konuşma pratiği sunuyoruz. Bu sayede, speaking confidence eksikliğini giderip, global toplantılara daha hazırlıklı hale gelmelerine yardımcı olabiliriz. 
 Size uygun bir zamanda detayları paylaşmak isterim.
 Saygılarımla,
@@ -2461,7 +2461,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -2534,7 +2534,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Merhaba İlker, HR profesyonelleri olarak iletişim becerilerinin önemini biliyoruz. Ekibinizin İngilizce konuşma güvenini artırmak, global toplantılara hazırlıklarını güçlendirmek için Konuşarak Öğren'in sunduğu çözümleri keşfetmek ister misiniz?</t>
+          <t>Merhaba Ilker Bey, HR profesyonelleri olarak iletişim becerilerinin önemini biliyoruz. Ekibinizin İngilizce konuşma güvenini artırmak, global toplantılara hazırlıklarını güçlendirmek için Konuşarak Öğren'in sunduğu çözümleri keşfetmek ister misiniz?</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
@@ -2566,12 +2566,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Doku Clinic</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2582,7 +2582,7 @@
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2622,18 +2622,18 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>85</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Merhaba Merve, gelişen global iş ortamında ekiplerinizin İngilizce konuşma pratiği yapma ihtiyacını göz önünde bulundurarak, Konuşarak Öğren olarak onlara nasıl destek olabileceğimizi paylaşmak isterim. Görüşmeye ne dersiniz?</t>
+          <t>Merhaba Merve Hanım, gelişen global iş ortamında ekiplerinizin İngilizce konuşma pratiği yapma ihtiyacını göz önünde bulundurarak, Konuşarak Öğren olarak onlara nasıl destek olabileceğimizi paylaşmak isterim. Görüşmeye ne dersiniz?</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
         <is>
           <t>Konu: Ekiplerinizin İngilizce Konuşma Becerilerini Geliştirin
-Merhaba Merve,
+Merhaba Merve Hanım,
 Umarım iyisinizdir. Gelişen global iş ortamında, çalışanlarınızın İngilizce konuşma pratiği yapma ihtiyacının ne denli önemli olduğunu biliyorum. Konuşarak Öğren olarak, ekiplerinize online İngilizce konuşma pratiği sunuyoruz. Böylece hem speaking confidence kazanabilirler hem de global toplantılara daha hazır hale gelebilirler.
 Detayları konuşmak için uygun bir zaman ayarlayabilir miyiz?
 Sevgiler,
@@ -2650,7 +2650,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -2662,12 +2662,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>ERNA MAŞ MAKİNA TİCARET VE SANAYİ A.Ş.</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2678,7 +2678,7 @@
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Çankırı, Turkey</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2718,18 +2718,18 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>Merhaba Mesut, insan kaynakları profesyonellerinin ekip iletişimini geliştirmelerine yardımcı olma konusunda uzmanız. Konuşarak Öğren olarak, çalışanlarınızın global toplantılara hazır olmalarını sağlamak için online İngilizce konuşma pratiği sunuyoruz. Detayları paylaşmak ister misiniz?</t>
+          <t>Merhaba Mesut Bey, insan kaynakları profesyonellerinin ekip iletişimini geliştirmelerine yardımcı olma konusunda uzmanız. Konuşarak Öğren olarak, çalışanlarınızın global toplantılara hazır olmalarını sağlamak için online İngilizce konuşma pratiği sunuyoruz. Detayları paylaşmak ister misiniz?</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
           <t>Konu: Çalışanlarınızın İletişim Becerilerini Geliştirin
-Merhaba Mesut,
+Merhaba Mesut Bey,
 Şirketinizde ekiplerinizi global toplantalara daha iyi hazırlamak ve İngilizce konuşma becerilerini geliştirmek için bir çözüm arıyorsanız, Konuşarak Öğren tam size göre. Online platformumuz sayesinde çalışanlarınız, güvenle iletişim kurma pratiği yapabilir. Gelin, ekiplerinizi daha etkili hale getirelim.
 Detayları görüşmek ister misiniz?
 İyi çalışmalar,
@@ -2743,7 +2743,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -2816,13 +2816,13 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Merhaba Ali, iletişim becerilerini geliştirmek ve çalışanların uluslararası toplantılara daha hazırlıklı olmalarını sağlamak için çözümler sunuyoruz. Konuşarak Öğren ile online İngilizce pratiği yaparak bu hedeflere ulaşmanızda yardımcı olabiliriz. Detayları görüşmek ister misin?</t>
+          <t>Merhaba Ali Bey, iletişim becerilerini geliştirmek ve çalışanların uluslararası toplantılara daha hazırlıklı olmalarını sağlamak için çözümler sunuyoruz. Konuşarak Öğren ile online İngilizce pratiği yaparak bu hedeflere ulaşmanızda yardımcı olabiliriz. Detayları görüşmek ister misin?</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
         <is>
           <t>Konu: Çalışanlarınızın İletişim Becerilerini Geliştirin
-Merhaba Ali,
+Merhaba Ali Bey,
 Kurumsal ekibinizin uluslararası ortamlarda daha etkili iletişim kurabilmesi için destek sunmak istiyoruz. Konuşarak Öğren, online İngilizce konuşma pratiği ile çalışanlarınızın kendine güvenini artırmayı ve global toplantılara hazır olmalarını sağlamayı hedefliyor. İlgilenirseniz, nasıl bir işbirliği yapabileceğimizi konuşmak isterim.
 İyi çalışmalar,
 [Adınız]</t>
@@ -2847,12 +2847,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Mavi</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2863,7 +2863,7 @@
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2903,18 +2903,18 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>95</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>Merhaba Ecem, HR profesyonellerinin ekip iletişimini güçlendirmek için arayış içinde olduğunu biliyorum. Konuşarak Öğren ile İngilizce konuşma pratiği yaparak, global toplantılara daha hazır hale gelmeleri konusunda nasıl yardımcı olabileceğimizi keşfetmek ister misin?</t>
+          <t>Merhaba Ecem Bey, HR profesyonellerinin ekip iletişimini güçlendirmek için arayış içinde olduğunu biliyorum. Konuşarak Öğren ile İngilizce konuşma pratiği yaparak, global toplantılara daha hazır hale gelmeleri konusunda nasıl yardımcı olabileceğimizi keşfetmek ister misin?</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
         <is>
           <t>Konu: Ekip İletişimini Güçlendirin
-Merhaba Ecem,
+Merhaba Ecem Bey,
 Ekiplerinizin İngilizce konuşma pratiği ile iletişim becerilerini geliştirmeleri, global toplantılarda daha özgüvenli olmalarını sağlayabilir. Konuşarak Öğren, kurumsal ekipler için özel olarak tasarlanmış online İngilizce programları sunuyor. Bu sayede, çalışanlarınızın gelişimini takip edebilir ve raporlarla destekleyebilirsiniz.
 Detayları konuşmak için bir görüşme ayarlayabilir miyiz?
 İyi çalışmalar,
@@ -2930,7 +2930,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -2942,12 +2942,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Cronton Design Hotel</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2958,7 +2958,7 @@
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2998,18 +2998,18 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>95</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>Merhaba Şeyda, HR profesyonellerinin ekiplerinin konuşma özgüvenini artırmalarına yardımcı olduğumuzu duydum. Global toplantılara hazırlık konusunda nasıl destek olabileceğimizi konuşmak ister misin?</t>
+          <t>Merhaba Şeyda Hanım, HR profesyonellerinin ekiplerinin konuşma özgüvenini artırmalarına yardımcı olduğumuzu duydum. Global toplantılara hazırlık konusunda nasıl destek olabileceğimizi konuşmak ister misin?</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
         <is>
           <t>Konu: Ekiplerinizin İngilizce Konuşma Gücünü Artırın
-Merhaba Şeyda,
+Merhaba Şeyda Hanım,
 Şirketinizdeki çalışanların İngilizce konuşma becerilerini geliştirmeleri, global toplantılarda daha etkili olmaları için kritik öneme sahip. Konuşarak Öğren, online İngilizce konuşma pratiğiyle ekip üyelerinizin güvenini artırarak, global arenada daha etkin olmalarına yardımcı olabilir.
 Gelişim takibi ve raporlama ile desteklenen programlarımız hakkında daha fazla bilgi almak istersen, sizinle görüşmeyi çok isterim.
 İyi çalışmalar,
@@ -3023,7 +3023,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -3035,12 +3035,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>İstanbul Beykent Üniversitesi</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3051,7 +3051,7 @@
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3091,18 +3091,18 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>95</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>Merhaba Mehmet, İngilizce konuşma pratiğiyle çalışanlarınızın özgüvenini artırmak ve uluslararası toplantılara hazırlıklarını güçlendirmek için nasıl bir yol izlediğinizi merak ediyorum. Bu konuda size yardımcı olabilecek bir çözüm sunabilirim. Görüşmek ister misiniz?</t>
+          <t>Merhaba Mehmet Bey, İngilizce konuşma pratiğiyle çalışanlarınızın özgüvenini artırmak ve uluslararası toplantılara hazırlıklarını güçlendirmek için nasıl bir yol izlediğinizi merak ediyorum. Bu konuda size yardımcı olabilecek bir çözüm sunabilirim. Görüşmek ister misiniz?</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
         <is>
           <t>Konu: Çalışanlarınızın İngilizce Konuşma Becerilerini Geliştirin
-Merhaba Mehmet,
+Merhaba Mehmet Bey,
 Kurumsal ekibinizin İngilizce konuşma becerilerini geliştirmek, uluslararası iletişimde daha etkili olmalarını sağlamak için önemli bir adım. Konuşarak Öğren olarak, çalışanlarınız için kişiselleştirilmiş online İngilizce konuşma pratiği sunuyoruz. Bu sayede, hem konuşma özgüvenleri artacak hem de global toplantılara hazırlıkları güçlenecek. 
 Detayları konuşmak için zaman ayırabilir miyiz? 
 Saygılarımla,
@@ -3118,7 +3118,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -3191,13 +3191,13 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Merhaba Serpil, global toplantılarda konuşma güveni ve farklı takımlarla etkili iletişim, HR profesyonelleri için kritik. Konuşarak Öğren'le, bu alandaki yetkinliğinizi artırabilirsiniz. Detaylar için bağlantıda kalalım!</t>
+          <t>Merhaba Serpil Bey, global toplantılarda konuşma güveni ve farklı takımlarla etkili iletişim, HR profesyonelleri için kritik. Konuşarak Öğren'le, bu alandaki yetkinliğinizi artırabilirsiniz. Detaylar için bağlantıda kalalım!</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
         <is>
           <t>Konu: HR Ekibiniz İçin İngilizce Konuşma Desteği
-Merhaba Serpil Hanım,
+Merhaba Serpil Bey,
 Şirketinizin uluslararası iletişimdeki başarıları için İngilizce konuşma pratiğinin önemini biliyoruz. Konuşarak Öğren, kurumsal ekiplere online İngilizce konuşma pratiği sunarak, global toplantılarda daha fazla özgüven ve etkili iletişim sağlamanıza yardımcı olabilir. Takım dinamiklerinizi güçlendirirken, gelişim takibi ve raporlama ile sürecinizi de destekliyoruz.
 Detayları paylaşmak için bir görüşme ayarlamayı çok isterim.
 Sevgiler,
@@ -3226,12 +3226,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>TÜBİTAK</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3242,7 +3242,7 @@
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Gebze, Kocaeli, Turkey</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3282,12 +3282,12 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Merhaba Ayten, Konuşarak Öğren olarak, çalışanlarınızın İngilizce konuşma pratiği yaparak global toplantılara daha hazır hale gelmelerine yardımcı olabiliriz. İlgilendiğiniz bir konu mu? Detayları paylaşmak isterim.</t>
+          <t>Merhaba Ayten Hanım, Konuşarak Öğren olarak, çalışanlarınızın İngilizce konuşma pratiği yaparak global toplantılara daha hazır hale gelmelerine yardımcı olabiliriz. İlgilendiğiniz bir konu mu? Detayları paylaşmak isterim.</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
@@ -3309,7 +3309,7 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -3321,12 +3321,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Blueforce</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3337,7 +3337,7 @@
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Başiskele, Kocaeli, Turkey</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -3377,18 +3377,18 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>95</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>Merhaba Sinem, İngilizce iletişim becerilerini geliştirmek ve çalışanların global toplantılara hazırlıklarını artırmak için online pratik sunuyoruz. Bu konuda daha fazla bilgi almak istersen, sevinirim! İyi çalışmalar dilerim.</t>
+          <t>Merhaba Sinem Hanım, İngilizce iletişim becerilerini geliştirmek ve çalışanların global toplantılara hazırlıklarını artırmak için online pratik sunuyoruz. Bu konuda daha fazla bilgi almak istersen, sevinirim! İyi çalışmalar dilerim.</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
         <is>
           <t>Konu: Çalışanlarınızın İngilizce Konuşma Becerilerini Geliştirme
-Merhaba Sinem,
+Merhaba Sinem Hanım,
 Kurumsal ekibinizin İngilizce konuşma pratiği ve global toplantılara hazırlık konusunda zorluklar yaşadığını biliyorum. Konuşarak Öğren olarak, online platformumuzda çalışanlarınıza kişiselleştirilmiş İngilizce pratik imkanı sunuyoruz. Gelişim takibi ve raporlama ile bu süreci daha etkili kılabiliriz. 
 Detayları paylaşmak ve size nasıl yardımcı olabileceğimizi konuşmak için bir görüşme ayarlamak ister misiniz?
 İyi çalışmalar,
@@ -3402,7 +3402,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -3414,12 +3414,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>COPRECI TR</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3430,7 +3430,7 @@
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Gebze, Kocaeli, Turkey</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3470,18 +3470,18 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>Merhaba İnci, HR profesyonellerine yönelik sunduğumuz online İngilizce konuşma pratiği ile ekiplerinizi toplantılarda daha özgüvenli hale getirebiliriz. Detayları paylaşmak ister misiniz?</t>
+          <t>Merhaba Inci Hanım, HR profesyonellerine yönelik sunduğumuz online İngilizce konuşma pratiği ile ekiplerinizi toplantılarda daha özgüvenli hale getirebiliriz. Detayları paylaşmak ister misiniz?</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
           <t>Konu: Ekibinizin İngilizce İletişim Becerilerini Geliştirin
-Merhaba İnci,
+Merhaba Inci Hanım,
 Şirketinizdeki HR süreçlerini güçlendirmek için, ekip üyelerinizin İngilizce iletişim becerilerini artırmaya yönelik özel online konuşma pratiği sunuyoruz. Bu program, çalışanlarınızın toplantılarda daha özgüvenli olmalarına ve etkin bir şekilde iletişim kurmalarına yardımcı olabilir. 
 Detayları konuşmak isterseniz, size yardımcı olmaktan memnuniyet duyarım.
 Saygılarımla,
@@ -3495,7 +3495,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -3507,12 +3507,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Cast Merkezi</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İK Yöneticisi</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -3523,7 +3523,7 @@
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -3563,12 +3563,12 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>90</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Merhaba Sevgi, kurumsal ekiplerin İngilizce konuşma pratiğiyle gelişimlerini destekleyen Konuşarak Öğren'i paylaşmak istedim. Çalışanlarınızın global toplantılarda daha özgüvenli olmalarına yardımcı olabiliriz. Görüşmek ister misiniz?</t>
+          <t>Merhaba Sevgi Hanım, kurumsal ekiplerin İngilizce konuşma pratiğiyle gelişimlerini destekleyen Konuşarak Öğren'i paylaşmak istedim. Çalışanlarınızın global toplantılarda daha özgüvenli olmalarına yardımcı olabiliriz. Görüşmek ister misiniz?</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -3660,13 +3660,13 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Merhaba Özgen, ekiplerin global toplantılara hazırlık sürecinde İngilizce konuşma becerilerini geliştirmek için nasıl bir yol izlediğinizi merak ettim. Konuşarak Öğren ile çalışanlarınızın kendine güvenini artırabiliriz. Detayları paylaşmak ister misiniz?</t>
+          <t>Merhaba Özgen Hanım, ekiplerin global toplantılara hazırlık sürecinde İngilizce konuşma becerilerini geliştirmek için nasıl bir yol izlediğinizi merak ettim. Konuşarak Öğren ile çalışanlarınızın kendine güvenini artırabiliriz. Detayları paylaşmak ister misiniz?</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
           <t>Konu: Ekiplerinizin Global Başarıları İçin İngilizce Pratiği
-Merhaba Özgen,
+Merhaba Özgen Hanım,
 Şirketinizdeki ekiplerin global toplantılara daha iyi hazırlanmaları için etkili bir yol arayışında olduğunuzu duydum. Konuşarak Öğren olarak, online İngilizce konuşma pratiği sunarak çalışanlarınızın kendine güvenini artırabiliriz. 
 Bu süreç, ekip üyelerinizin iletişim becerilerini geliştirmelerine ve uluslararası iş ortamında daha etkili olmalarına yardımcı olacaktır. Detayları konuşmak için bir zaman ayıralım mı?
 Saygılarımla,
@@ -3754,13 +3754,13 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>Merhaba Müzeyyen, HR alanındaki deneyiminizle global iş ortamında etkili iletişimin önemini bildiğinizi düşünüyorum. Kurumsal ekiplerdeki İngilizce konuşma becerilerini geliştirmek için bir çözüm sunuyoruz. Detayları paylaşmak isterim.</t>
+          <t>Merhaba Müzeyyen Hanım, HR alanındaki deneyiminizle global iş ortamında etkili iletişimin önemini bildiğinizi düşünüyorum. Kurumsal ekiplerdeki İngilizce konuşma becerilerini geliştirmek için bir çözüm sunuyoruz. Detayları paylaşmak isterim.</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
         <is>
           <t>Konu: Ekip İletişimini Güçlendirin
-Merhaba Müzeyyen,
+Merhaba Müzeyyen Hanım,
 Kurumsal ekiplerde çalışanların İngilizce konuşma becerilerini geliştirmek, global işbirliğini artırabilir. Konuşarak Öğren olarak, çevrimiçi platformda personelinizin konuşma pratiği yapmasını sağlıyoruz. Bu süreç, gelişim takibi ve raporlama ile destekleniyor. Ekibinizin güvenle global toplantılara katılmasına yardımcı olmak için bir görüşme ayarlamak ister misiniz?
 Saygılarımla,
 [İsminiz]</t>
@@ -3785,12 +3785,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>İMED</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -3801,7 +3801,7 @@
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -3841,18 +3841,18 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>95</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>Merhaba Şule, kurumsal ekiplerin İngilizce iletişim becerilerini geliştirme üzerine çalıştığınızı biliyorum. Konuşarak Öğren ile, çalışanlarınızın global toplantılara daha iyi hazırlanmasını sağlamak için bir çözüm sunuyoruz. Detayları paylaşmak ister misiniz?</t>
+          <t>Merhaba Şule Hanım, kurumsal ekiplerin İngilizce iletişim becerilerini geliştirme üzerine çalıştığınızı biliyorum. Konuşarak Öğren ile, çalışanlarınızın global toplantılara daha iyi hazırlanmasını sağlamak için bir çözüm sunuyoruz. Detayları paylaşmak ister misiniz?</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
           <t>Konu: İngilizce İletişim Becerilerini Geliştirin
-Merhaba Şule,
+Merhaba Şule Hanım,
 Gelişen global iş ortamında, çalışanlarınızın İngilizce iletişim becerilerini artırmak adına etkili bir çözüm arayışında olduğunuzu biliyorum. Konuşarak Öğren, kurumsal ekipler için online İngilizce konuşma pratiği, gelişim takibi ve raporlama hizmeti sunuyor. Ekibinizin global toplantılara daha iyi hazırlanmalarına destek olmak ve konuşma güvenlerini artırmak için birlikte çalışabiliriz. Detayları görüşmek ister misiniz?
 Sevgiler,
 [Adınız]</t>
@@ -3865,7 +3865,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -3877,12 +3877,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>ELSAN Elektrik Sanayi ve Ticaret A.Ş.</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -3893,7 +3893,7 @@
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Ankara, Turkey</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -3933,18 +3933,18 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>95</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>Merhaba Zeynep, çalışanların global toplantılarda daha etkili iletişim kurabilmesi için online İngilizce konuşma pratiği sunuyoruz. Ekibinizin kendine güvenini artırmak ve iletişim becerilerini geliştirmek için birlikte çalışabiliriz. Görüşmek ister misiniz?</t>
+          <t>Merhaba Zeynep Hanım, çalışanların global toplantılarda daha etkili iletişim kurabilmesi için online İngilizce konuşma pratiği sunuyoruz. Ekibinizin kendine güvenini artırmak ve iletişim becerilerini geliştirmek için birlikte çalışabiliriz. Görüşmek ister misiniz?</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
         <is>
           <t>Konu: Global İletişim Becerilerini Geliştirin
-Merhaba Zeynep,
+Merhaba Zeynep Hanım,
 Kurumsal ekibinizin global toplantılarda daha etkili olabilmesi için iletişim becerilerini geliştirmek önemlidir. Konuşarak Öğren olarak, online İngilizce konuşma pratiği ve gelişim takibi sunuyoruz. Çalışanlarınızın kendine güvenini artırarak, global iş dünyasında daha hazır hale gelmelerine yardımcı olabiliriz. İlgilenirseniz, detayları paylaşmak isterim.
 İyi çalışmalar,
 [Adınız]</t>
@@ -3957,7 +3957,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -3969,12 +3969,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Parex</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -3985,7 +3985,7 @@
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -4025,18 +4025,18 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>Merhaba Bahar, ekibinizin İngilizce iletişim becerilerini geliştirmek için online konuşma pratiği sunuyoruz. Küresel etkileşimlerde daha özgüvenli bir iletişim için nasıl yardımcı olabileceğimizi konuşmak ister misiniz?</t>
+          <t>Merhaba Bahar Hanım, ekibinizin İngilizce iletişim becerilerini geliştirmek için online konuşma pratiği sunuyoruz. Küresel etkileşimlerde daha özgüvenli bir iletişim için nasıl yardımcı olabileceğimizi konuşmak ister misiniz?</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
         <is>
           <t>Konu: İngilizce İletişim Becerilerinizi Geliştirin
-Merhaba Bahar,
+Merhaba Bahar Hanım,
 Şirketinizdeki ekip üyelerinin İngilizce iletişim becerilerini geliştirmek ve global etkileşimlerde daha etkili olmalarına yardımcı olmak için online İngilizce konuşma pratiği sunuyoruz. Gelişim takibi ve raporlama ile süreçlerinizi kolaylaştırıyoruz. Ekiplerinizin daha özgüvenli olmasını sağlayacak çözümlerimiz hakkında daha fazla bilgi almak isterseniz, sizinle görüşmek isterim.
 İyi çalışmalar,
 [Adınız]
@@ -4051,7 +4051,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -4063,12 +4063,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Kalyon PV</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -4079,7 +4079,7 @@
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Ankara, Turkey</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -4119,7 +4119,7 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>95</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
@@ -4146,7 +4146,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -4219,13 +4219,13 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>Merhaba İlker, HR alanında çalışan biri olarak, kurumsal ekiplerin İngilizce iletişim becerilerini geliştirmeleri konusunda önemli bir rol oynadığınızı biliyorum. Konuşarak Öğren ile bu becerileri güçlendirmek ve global toplantılara hazırlık sağlamak üzerine bir görüşme yapmayı ister misiniz?</t>
+          <t>Merhaba Ilker Bey, HR alanında çalışan biri olarak, kurumsal ekiplerin İngilizce iletişim becerilerini geliştirmeleri konusunda önemli bir rol oynadığınızı biliyorum. Konuşarak Öğren ile bu becerileri güçlendirmek ve global toplantılara hazırlık sağlamak üzerine bir görüşme yapmayı ister misiniz?</t>
         </is>
       </c>
       <c r="P41" t="inlineStr">
         <is>
           <t>Konu: Kurumsal Ekipler İçin İngilizce Pratiği
-Merhaba İlker,
+Merhaba Ilker Bey,
 Umarım iyisinizdir. Şirketinizdeki ekiplerin global toplantılara daha iyi hazırlanmaları ve İngilizce konuşma konusundaki güvenlerini artırmaları için online pratik fırsatları sunuyoruz. Konuşarak Öğren ile, ekip üyelerinizin iletişim becerilerini geliştirmek ve gelişimlerini raporlamak mümkün. Sizinle bu konuda bir görüşme yapmayı çok isterim.
 İyi günler dilerim,
 [Adınız]  
@@ -4253,12 +4253,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Kopuz Şirketler Grubu</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>Grup İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -4269,7 +4269,7 @@
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -4309,18 +4309,18 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>Merhaba Gökçe, HR alanında çalışan bir profesyonel olarak, çalışanların İngilizce konuşma becerilerini geliştirmelerine nasıl katkıda bulunduğunuzu merak ediyorum. Konuşarak Öğren ile bu konuda destek olabiliriz. Görüşmek ister misiniz?</t>
+          <t>Merhaba Gökçe Hanım, HR alanında çalışan bir profesyonel olarak, çalışanların İngilizce konuşma becerilerini geliştirmelerine nasıl katkıda bulunduğunuzu merak ediyorum. Konuşarak Öğren ile bu konuda destek olabiliriz. Görüşmek ister misiniz?</t>
         </is>
       </c>
       <c r="P42" t="inlineStr">
         <is>
           <t>Konu: Çalışanlarınızın İletişim Becerilerini Geliştirin
-Merhaba Gökçe,
+Merhaba Gökçe Hanım,
 Kurumsal ekibinizin İngilizce konuşma pratiği yaparak global toplantılara daha hazır hale gelmesine nasıl katkıda bulunabileceğimizi konuşmak isterim. Konuşarak Öğren, çalışanlarınızın iletişim becerilerini geliştirmelerine ve güvenle konuşmalarına yardımcı oluyor. Eğitim süreçlerinize entegre edebileceğimiz çözümler sunuyoruz. İlgilenirseniz, detayları görüşmek için bir zaman ayarlayalım.
 İyi çalışmalar,
 [Adınız]</t>
@@ -4333,7 +4333,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -4406,13 +4406,13 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>Merhaba İlker Bey, iletişim becerileri geliştirmek, çalışanlarınızın global toplantılara hazırlığını artırmak için Konuşarak Öğren olarak destek olabileceğimizi düşünüyorum. Daha fazla bilgi almak ister misiniz?</t>
+          <t>Merhaba Ilker Bey, iletişim becerileri geliştirmek, çalışanlarınızın global toplantılara hazırlığını artırmak için Konuşarak Öğren olarak destek olabileceğimizi düşünüyorum. Daha fazla bilgi almak ister misiniz?</t>
         </is>
       </c>
       <c r="P43" t="inlineStr">
         <is>
           <t>Konu: Çalışanlarınızın İletişim Becerilerini Geliştirin
-Merhaba İlker Bey,
+Merhaba Ilker Bey,
 Şirketinizdeki çalışanların İngilizce konuşma becerilerini geliştirmek ve global toplantılara hazırlıklarını artırmak adına Konuşarak Öğren olarak size yardımcı olabiliriz. Online platformumuzla, çalışanlarınızın iletişim yeteneklerini güçlendirirken gelişim takibi ve raporlama sunuyoruz. Daha fazla bilgi almak isterseniz, sizinle görüşmekten memnuniyet duyarım.
 İyi çalışmalar,
 [Adınız]</t>
@@ -4437,12 +4437,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Kibar Holding</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>HRBP Müdürü</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -4453,7 +4453,7 @@
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -4493,12 +4493,12 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>Merhaba Lale, İngilizce iletişim becerilerini güçlendirmek ve ekiplerinizi uluslararası toplantalara hazırlamak için online konuşma pratiği sunuyoruz. Detayları paylaşmak isterim. Görüşmek üzere!</t>
+          <t>Merhaba Lale Hanım, İngilizce iletişim becerilerini güçlendirmek ve ekiplerinizi uluslararası toplantalara hazırlamak için online konuşma pratiği sunuyoruz. Detayları paylaşmak isterim. Görüşmek üzere!</t>
         </is>
       </c>
       <c r="P44" t="inlineStr">
@@ -4518,7 +4518,7 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -4530,12 +4530,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Optimum İnsan Kaynakları</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>Senior Human Resources Specialist</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -4546,7 +4546,7 @@
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -4586,18 +4586,18 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>Merhaba Gizem, global toplantılarda etkili iletişimin ne kadar önemli olduğunu biliyoruz. Ekibinizin İngilizce konuşma pratiği yaparak kendine güven kazanmasına yardımcı olabiliriz. Daha fazla bilgi almak isterseniz, memnuniyetle konuşalım!</t>
+          <t>Merhaba Gizem Hanım, global toplantılarda etkili iletişimin ne kadar önemli olduğunu biliyoruz. Ekibinizin İngilizce konuşma pratiği yaparak kendine güven kazanmasına yardımcı olabiliriz. Daha fazla bilgi almak isterseniz, memnuniyetle konuşalım!</t>
         </is>
       </c>
       <c r="P45" t="inlineStr">
         <is>
           <t>Konu: İletişim Becerilerinizi Geliştirin
-Merhaba Gizem,
+Merhaba Gizem Hanım,
 Global toplantılarda etkili iletişim, ekiplerin başarısını doğrudan etkiler. Konuşarak Öğren olarak, şirketinizin İngilizce konuşma pratiği yaparak çalışanlarınızın kendine güven kazanmasına yardımcı olabiliriz. Ekip üyelerinin gelişimini takip edebilir ve raporlayabiliriz. Bu konuyu daha detaylı konuşmak için bir görüşme ayarlamayı ister misiniz?
 Saygılarımla,
 [Adınız]
@@ -4611,7 +4611,7 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -4718,12 +4718,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Yardımcı Beton</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -4734,7 +4734,7 @@
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Konya, Turkey</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -4774,18 +4774,18 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>95</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>Merhaba Şahika, global HR rollerinde iletişim becerilerinin önemini biliyorum. Konuşarak Öğren ile online İngilizce pratiği yaparak ekibinizin global toplantılara daha hazır olmasını sağlayabilirsiniz. Detayları paylaşmak isterim.</t>
+          <t>Merhaba Şahika Hanım, global HR rollerinde iletişim becerilerinin önemini biliyorum. Konuşarak Öğren ile online İngilizce pratiği yaparak ekibinizin global toplantılara daha hazır olmasını sağlayabilirsiniz. Detayları paylaşmak isterim.</t>
         </is>
       </c>
       <c r="P47" t="inlineStr">
         <is>
           <t>Konu: Global HR İletişim Becerilerinizi Geliştirin
-Merhaba Şahika,
+Merhaba Şahika Hanım,
 Şirketinizdeki HR profesyonellerinin İngilizce iletişim becerilerini geliştirmek, uluslararası işbirliklerinde başarıyı artırabilir. Konuşarak Öğren, kurumsal ekiplerinize online konuşma pratiği sunarak, global toplantılara daha hazır olmalarını sağlıyor. Ekibinizin bu fırsattan nasıl faydalanabileceğini konuşmak ister misiniz?
 Saygılarımla,
 [Adınız]</t>
@@ -4798,7 +4798,7 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -4810,12 +4810,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>ANL FOOD INC</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -4826,7 +4826,7 @@
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -4866,18 +4866,18 @@
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>Merhaba Ezgi, Konuşarak Öğren ile ekiplerinizi küresel toplantılara daha hazır hale getirebilirsiniz. İngilizce konuşma pratiği ile iletişim becerilerini geliştirmek ve güven artırmak için bir görüşme ayarlamak ister misiniz?</t>
+          <t>Merhaba Ezgi Hanım, Konuşarak Öğren ile ekiplerinizi küresel toplantılara daha hazır hale getirebilirsiniz. İngilizce konuşma pratiği ile iletişim becerilerini geliştirmek ve güven artırmak için bir görüşme ayarlamak ister misiniz?</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
         <is>
           <t>Konu: Ekip İletişimini Güçlendirin
-Merhaba Ezgi,
+Merhaba Ezgi Hanım,
 Kurumsal ekibinizin global toplantılardaki iletişimini geliştirmek için etkili bir çözüm arıyorsanız, Konuşarak Öğren tam size göre. Online İngilizce konuşma pratiği ile ekip üyelerinizin konuşma güvenini artırabilir ve toplantılara daha iyi hazırlanmış olmalarını sağlayabilirsiniz. 
 Eğitim programlarımız hakkında daha fazla bilgi almak isterseniz, size yardımcı olmaktan memnuniyet duyarım.
 Saygılarımla,
@@ -4894,7 +4894,7 @@
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -4906,12 +4906,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>BÜROTIME</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -4922,7 +4922,7 @@
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -4962,18 +4962,18 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>95</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>Merhaba Onur, İngilizce konuşma becerileri global iş dünyasında büyük önem taşıyor. Konuşarak Öğren, ekiplerinize çevrimiçi pratik yapma imkanı sunarak güvenlerini artırmalarına yardımcı olabilir. Görüşmek ister misiniz?</t>
+          <t>Merhaba Onur Bey, İngilizce konuşma becerileri global iş dünyasında büyük önem taşıyor. Konuşarak Öğren, ekiplerinize çevrimiçi pratik yapma imkanı sunarak güvenlerini artırmalarına yardımcı olabilir. Görüşmek ister misiniz?</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
         <is>
           <t>Konu: Ekiplerinizin İngilizce Konuşma Becerilerini Geliştirin
-Merhaba Onur,
+Merhaba Onur Bey,
 Kurumsal ekipler için İngilizce konuşma pratiği sağlamak, global iş ortamlarında iletişim becerilerini güçlendirmenin anahtarı. Konuşarak Öğren olarak, çalışanlarınızın konuşma güvenini artırmalarına ve uluslararası toplantılara hazırlanmalarına yardımcı oluyoruz. Ekiplerinize özel programlarımızla gelişim takibi ve raporlama sunuyoruz. Detayları paylaşmak için bir görüşme ayarlayabilir miyiz?
 Saygılarımla,
 [Adınız]</t>
@@ -4986,7 +4986,7 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -4998,12 +4998,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Aran Tekstil San. Tic. A.Ş.</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -5014,7 +5014,7 @@
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Denizli, Turkey</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -5054,18 +5054,18 @@
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>95</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>Merhaba Serdal, HR ekiplerinin iletişim becerilerini geliştirmesine yardımcı olan etkili bir çözüm sunuyoruz. Küresel toplantılarda daha fazla özgüven ve etkili iletişim için konuşma pratiği yapmayı düşünür müsünüz? Detayları paylaşmak isterim.</t>
+          <t>Merhaba Serdal Bey, HR ekiplerinin iletişim becerilerini geliştirmesine yardımcı olan etkili bir çözüm sunuyoruz. Küresel toplantılarda daha fazla özgüven ve etkili iletişim için konuşma pratiği yapmayı düşünür müsünüz? Detayları paylaşmak isterim.</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
         <is>
           <t>Konu: Küresel Toplantılarda Başarı İçin Konuşma Pratiği
-Merhaba Serdal,
+Merhaba Serdal Bey,
 Kurumsal ekibinizin global toplantılarda daha etkili iletişim kurabilmesi için bir çözüm sunmak istiyorum. Konuşarak Öğren, çalışanlarınıza online İngilizce konuşma pratiği ve gelişim takibi sunarak, kendilerine olan güvenlerini artırmalarını sağlıyor. Bu sayede, ekibinizin uluslararası platformlarda daha başarılı olmasını hedefliyoruz.
 Detayları görüşmek isterseniz, sevinirim.
 İyi çalışmalar,
@@ -5079,7 +5079,7 @@
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -5091,12 +5091,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Dicle FZA Otomotiv San. Ve Tic. A.Ş.</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>Satın Alma ve Personel Müdürü</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -5107,7 +5107,7 @@
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -5147,18 +5147,18 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>95</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>Merhaba Türkan, HR profesyonelleri için global toplantılarda etkili iletişim önemli. Konuşarak Öğren ile ekiplerinizin İngilizce konuşma pratiğini destekleyerek bu alanda güven kazanmalarına yardımcı olabiliriz. Detayları paylaşmayı çok isterim.</t>
+          <t>Merhaba Türkan Bey, HR profesyonelleri için global toplantılarda etkili iletişim önemli. Konuşarak Öğren ile ekiplerinizin İngilizce konuşma pratiğini destekleyerek bu alanda güven kazanmalarına yardımcı olabiliriz. Detayları paylaşmayı çok isterim.</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
         <is>
           <t>Konu: Ekip İletişimini Güçlendirin
-Merhaba Türkan, 
+Merhaba Türkan Bey, 
 Ekiplerinizin global toplantılarda daha etkili iletişim kurabilmesi için İngilizce konuşma becerilerini geliştirmek önemli. Konuşarak Öğren, çalışanlarınızın konuşma pratiği yapmasını ve gelişimlerini takip etmesini sağlıyor. Eğlenceli ve etkileşimli bir ortamda, ekibinizin kendine güvenini artırmak için nasıl bir yol izleyebileceğimizi konuşmak isterim.
 İlgilenirseniz, bir görüşme ayarlayalım. 
 İyi çalışmalar,
@@ -5172,7 +5172,7 @@
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -5184,12 +5184,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Remed Assistance</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -5200,7 +5200,7 @@
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -5240,12 +5240,12 @@
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>85</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>Merhaba Ezgi, İngilizce konuşma pratiği ile ekiplerinizi global toplantılara daha hazır hale getirmek için birlikte çalışabileceğimizi düşünüyorum. Konuşarak Öğren ile çalışanlarımızın özgüvenini artırabiliriz. Detayları konuşmak ister misiniz?</t>
+          <t>Merhaba Ezgi Hanım, İngilizce konuşma pratiği ile ekiplerinizi global toplantılara daha hazır hale getirmek için birlikte çalışabileceğimizi düşünüyorum. Konuşarak Öğren ile çalışanlarımızın özgüvenini artırabiliriz. Detayları konuşmak ister misiniz?</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -5276,12 +5276,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>İstanbul Silah ve Savunma Sanayi A.Ş.</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -5292,7 +5292,7 @@
       <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -5332,12 +5332,12 @@
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>85</t>
         </is>
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>Merhaba Duygu, LinkedIn profilinizdeki HR deneyiminizi inceledim. Kurumsal ekiplerdeki İngilizce konuşma becerilerini geliştirmek için sizinle bağlantı kurmak istedim. Global toplantılara hazırlık sağlamak, çalışanlarınızın güvenini artırabilir. Görüşmek ister misiniz?</t>
+          <t>Merhaba Duygu Hanım, LinkedIn profilinizdeki HR deneyiminizi inceledim. Kurumsal ekiplerdeki İngilizce konuşma becerilerini geliştirmek için sizinle bağlantı kurmak istedim. Global toplantılara hazırlık sağlamak, çalışanlarınızın güvenini artırabilir. Görüşmek ister misiniz?</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -5358,7 +5358,7 @@
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -5431,13 +5431,13 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>Merhaba Izel, HR alanındaki deneyiminizle, ekipler arası iletişimi güçlendirmenin önemini biliyorsunuz. Konuşarak Öğren ile online İngilizce pratiği yaparak, ekiplerinizin küresel toplantılara daha hazır hale gelmesine yardımcı olabiliriz. Detayları paylaşmak ister misiniz?</t>
+          <t>Merhaba Izel Bey, HR alanındaki deneyiminizle, ekipler arası iletişimi güçlendirmenin önemini biliyorsunuz. Konuşarak Öğren ile online İngilizce pratiği yaparak, ekiplerinizin küresel toplantılara daha hazır hale gelmesine yardımcı olabiliriz. Detayları paylaşmak ister misiniz?</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
         <is>
           <t>Konu: Takım İletişimini Güçlendirin
-Merhaba Izel,
+Merhaba Izel Bey,
 HR alanındaki deneyiminizle, çalışanların iletişim becerilerinin artmasının ekip dinamiklerine katkısını biliyorsunuzdur. Konuşarak Öğren, kurumsal ekiplerinize online İngilizce konuşma pratiği sunarak, global toplantılara hazırlık ve gelişim takibi yapmanızı sağlıyor. Ekibinizin kendine güvenle iletişim kurabilmesi için nasıl bir destek sunabileceğimizi konuşmak ister misiniz?
 Saygılarımla,
 [Adınız]</t>
@@ -5462,12 +5462,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>İmza</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -5478,7 +5478,7 @@
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -5518,18 +5518,18 @@
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>Merhaba Yasemin, gelişen global iş ortamında çalışanların İngilizce konuşma becerilerini artırmanın öneminin farkındayım. Konuşarak Öğren olarak, kurumsal ekiplerin speaking confidence ve global meeting readiness alanlarında gelişim sağlamalarına yardımcı olabiliyoruz. Görüşmek ister misin?</t>
+          <t>Merhaba Yasemin Hanım, gelişen global iş ortamında çalışanların İngilizce konuşma becerilerini artırmanın öneminin farkındayım. Konuşarak Öğren olarak, kurumsal ekiplerin speaking confidence ve global meeting readiness alanlarında gelişim sağlamalarına yardımcı olabiliyoruz. Görüşmek ister misin?</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
         <is>
           <t>Konu: İngilizce Konuşma Pratiği ile Ekibinizi Güçlendirin
-Merhaba Yasemin,
+Merhaba Yasemin Hanım,
 Kurumsal ekipler için İngilizce konuşma pratiği sağlamak, gelişen global iş ortamında önemli bir ihtiyaç haline geldi. Konuşarak Öğren olarak, ekiplerinizin speaking confidence ve global meeting readiness alanlarında gelişim göstermelerine yardımcı oluyoruz.
 Eğer şirketinizin bu alanda destek alabileceği bir çözüm arayışı varsa, sizinle bu konuyu daha detaylı konuşmak isterim. Uygun olduğunuz bir zaman diliminde görüşebilir miyiz?
 İyi çalışmalar,
@@ -5543,7 +5543,7 @@
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -5647,12 +5647,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Bursa Çimento Fabrikası A.Ş.</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -5663,7 +5663,7 @@
       <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Bursa, Turkey</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -5703,18 +5703,18 @@
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>95</t>
         </is>
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>Merhaba Orhan, İngilizce iletişimde güven eksikliği, global toplantılara hazırlık açısından büyük bir engel olabilir. Kurumsal ekipler için online konuşma pratiği sunuyoruz. Bu konuda bir konuşma ayarlamak ister misiniz?</t>
+          <t>Merhaba Orhan Bey, İngilizce iletişimde güven eksikliği, global toplantılara hazırlık açısından büyük bir engel olabilir. Kurumsal ekipler için online konuşma pratiği sunuyoruz. Bu konuda bir konuşma ayarlamak ister misiniz?</t>
         </is>
       </c>
       <c r="P57" t="inlineStr">
         <is>
           <t>Konu: Global Toplantılara Hazırlık İçin İngilizce Pratiği
-Merhaba Orhan Çelebi,
+Merhaba Orhan Bey Çelebi,
 Umarım bu mesajım sizi iyi bulur. Şirketinizdeki ekiplerin İngilizce iletişiminde yaşadığı güven eksikliği, global toplantılarda zorlanmalara neden olabilir. Konuşarak Öğren olarak, ekiplerinize online İngilizce konuşma pratiği sunarak bu sorunu aşmalarına yardımcı olabiliriz. Gelişim takibi ve raporlama ile desteklenen programlarımız, ekiplerinizin kendine güvenini artırmalarını sağlayacaktır. 
 Daha fazla bilgi almak veya bir toplantı ayarlamak isterseniz, lütfen benimle iletişime geçin.
 Saygılarımla,
@@ -5728,7 +5728,7 @@
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -5801,7 +5801,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>Merhaba H Özdemir, global toplantılarda çalışanlarınızın İngilizce konuşma güvenini artırmak için neler yaptığınızı merak ediyorum. Konuşarak Öğren, online pratik ve gelişim takibi ile bu konuda destek olabilir. Görüşmek ister misiniz?</t>
+          <t>Merhaba H Bey Özdemir, global toplantılarda çalışanlarınızın İngilizce konuşma güvenini artırmak için neler yaptığınızı merak ediyorum. Konuşarak Öğren, online pratik ve gelişim takibi ile bu konuda destek olabilir. Görüşmek ister misiniz?</t>
         </is>
       </c>
       <c r="P58" t="inlineStr">
@@ -5833,12 +5833,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Karaca Gümrük Müşavirliği</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -5849,7 +5849,7 @@
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -5889,7 +5889,7 @@
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>95</t>
         </is>
       </c>
       <c r="O59" t="inlineStr">
@@ -5914,7 +5914,7 @@
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -5926,12 +5926,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Oxigen Laboratuvarları</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Yöneticisi</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -5942,7 +5942,7 @@
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -5982,18 +5982,18 @@
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>95</t>
         </is>
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>Merhaba Derya, İngilizce konuşma pratiği ile çalışanların kendine güvenini artırmak ve global toplantılara hazırlık konusunda destek olabileceğimizi düşünmüştüm. Konuşarak Öğren'i keşfetmek isterseniz, memnuniyetle paylaşırım. İyi çalışmalar dilerim!</t>
+          <t>Merhaba Derya Hanım, İngilizce konuşma pratiği ile çalışanların kendine güvenini artırmak ve global toplantılara hazırlık konusunda destek olabileceğimizi düşünmüştüm. Konuşarak Öğren'i keşfetmek isterseniz, memnuniyetle paylaşırım. İyi çalışmalar dilerim!</t>
         </is>
       </c>
       <c r="P60" t="inlineStr">
         <is>
           <t>Konu: Çalışanlarınızın İngilizce Konuşma Becerilerini Geliştirin
-Merhaba Derya,
+Merhaba Derya Hanım,
 Şirketinizdeki çalışanların İngilizce konuşma güvenini artırmak ve global toplantılara hazırlık süreçlerini desteklemek için online pratik imkanı sunuyoruz. Konuşarak Öğren, gelişim takibi ve raporlama ile süreci daha etkili hale getiriyor. 
 İlgilenirseniz, detayları paylaşmaktan memnuniyet duyarım.
 İyi çalışmalar,
@@ -6009,7 +6009,7 @@
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -6021,12 +6021,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>GDZ Elektrik Dağıtım</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -6037,7 +6037,7 @@
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>İzmir, Turkey</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -6077,18 +6077,18 @@
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>Merhaba Özge, kurumsal ekiplerde İngilizce konuşma pratiği ve güven eksikliğini gidermeye yönelik çözümler sunuyoruz. Çalışanlarınızın global toplantılara daha hazır hale gelmesi için birlikte çalışmayı çok isterim. Detayları konuşalım mı?</t>
+          <t>Merhaba Özge Hanım, kurumsal ekiplerde İngilizce konuşma pratiği ve güven eksikliğini gidermeye yönelik çözümler sunuyoruz. Çalışanlarınızın global toplantılara daha hazır hale gelmesi için birlikte çalışmayı çok isterim. Detayları konuşalım mı?</t>
         </is>
       </c>
       <c r="P61" t="inlineStr">
         <is>
           <t>Konu: Çalışanlarınızın İngilizce Konuşma Becerilerini Geliştirin
-Merhaba Özge,
+Merhaba Özge Hanım,
 Umarım iyisinizdir! Kurumsal ekiplerde İngilizce konuşma pratiği ve güven eksikliği, global toplantılarda etkili iletişim için önemli bir engel oluşturabiliyor. Konuşarak Öğren olarak, ekiplerinize online İngilizce konuşma pratiği sunarak, bu konuda gelişimlerini takip etmenize yardımcı olabiliriz. Çalışanlarınızın speaking confidence’ını artırarak, global toplantılara daha hazır olmalarını sağlamak için bir araya gelmeyi çok isterim.
 Görüşmek dileğiyle,
 [Adınız]</t>
@@ -6101,7 +6101,7 @@
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -6113,12 +6113,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Gökçelik A.Ş.</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -6129,7 +6129,7 @@
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Bursa, Turkey</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -6169,18 +6169,18 @@
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>90</t>
         </is>
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>Merhaba Melike, HR alanında çalışan bir profesyonel olarak, kurumsal ekiplerin İngilizce konuşma pratiğini geliştirmesi konusunda nasıl destek sağlayabileceğimizi konuşmak isterim. Konuşarak Öğren ile çalışanlarınızın güvenle konuşmasını sağlamak mümkün. Görüşmek dileğiyle!</t>
+          <t>Merhaba Melike Hanım, HR alanında çalışan bir profesyonel olarak, kurumsal ekiplerin İngilizce konuşma pratiğini geliştirmesi konusunda nasıl destek sağlayabileceğimizi konuşmak isterim. Konuşarak Öğren ile çalışanlarınızın güvenle konuşmasını sağlamak mümkün. Görüşmek dileğiyle!</t>
         </is>
       </c>
       <c r="P62" t="inlineStr">
         <is>
           <t>Konu: İngilizce Konuşma Pratiği ile Güçlü Ekipler Yaratın
-Merhaba Melike,
+Merhaba Melike Hanım,
 Kurumsal ekibinizin global iletişimde daha etkili olabilmesi için İngilizce konuşma pratiği sunan Konuşarak Öğren’i tanıtmak istiyorum. Çalışanlarınızın konuşma güvenini artırarak toplantılara daha hazır hale gelmelerini sağlayabiliriz. Detayları görüşmek ister misiniz?
 Saygılarımla,
 [Adınız]</t>
@@ -6193,7 +6193,7 @@
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -6266,13 +6266,13 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>Merhaba Deniz, İngilizce konuşma pratiği ile çalışanların global toplantılardaki özgüvenini artırmanıza yardımcı olabiliriz. Kurumsal ekibinizin performansını artırmak için birlikte çalışmayı çok isteriz. Detayları konuşalım! Sevgiler, Konuşarak Öğren.</t>
+          <t>Merhaba Deniz Hanım, İngilizce konuşma pratiği ile çalışanların global toplantılardaki özgüvenini artırmanıza yardımcı olabiliriz. Kurumsal ekibinizin performansını artırmak için birlikte çalışmayı çok isteriz. Detayları konuşalım! Sevgiler, Konuşarak Öğren.</t>
         </is>
       </c>
       <c r="P63" t="inlineStr">
         <is>
           <t>Konu: Çalışanlarınızın İngilizce Konuşma Yetkinliğini Artırın
-Merhaba Deniz,
+Merhaba Deniz Hanım,
 HR alanındaki tecrübenizle, global toplantılarda çalışanların özgüvenini artırmanın önemini biliyorsunuzdur. Konuşarak Öğren olarak, kurumsal ekiplere yönelik online İngilizce konuşma pratiği sunuyoruz. Çalışanlarınızın iletişim becerilerini geliştirerek, hem katılımlarını hem de performanslarını artırabiliriz. Sizinle bu konuda detaylı bir görüşme yapmak isterim.
 Sevgiler,
 [Adınız]  
@@ -6298,12 +6298,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>EMSA Generator</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Yöneticisi</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -6314,7 +6314,7 @@
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -6354,18 +6354,18 @@
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>Merhaba Murat, HR alanındaki deneyiminizle ekibinizin global toplantılardaki iletişimini güçlendirmek için bir çözüm sunmak istiyorum. Online İngilizce konuşma pratiği ile ekip üyelerinizin özgüvenini artırabiliriz. Detayları paylaşmak ister misiniz?</t>
+          <t>Merhaba Murat Bey, HR alanındaki deneyiminizle ekibinizin global toplantılardaki iletişimini güçlendirmek için bir çözüm sunmak istiyorum. Online İngilizce konuşma pratiği ile ekip üyelerinizin özgüvenini artırabiliriz. Detayları paylaşmak ister misiniz?</t>
         </is>
       </c>
       <c r="P64" t="inlineStr">
         <is>
           <t>Konu: Global Toplantılarda İletişim Gücünüzü Artırın
-Merhaba Murat,
+Merhaba Murat Bey,
 HR profesyoneli olarak, ekibinizin global toplantılarda etkili iletişim kurma yetkinliğini artırmak istediğinizi biliyorum. Konuşarak Öğren olarak, kurumsal ekipler için kişiselleştirilmiş online İngilizce konuşma pratiği sunuyoruz. Bu sayede çalışanlarınızın kendilerine olan güvenlerini artırarak, uluslararası ortamlarda daha etkili olmalarını sağlıyoruz.
 İlgilenirseniz, detayları konuşmak için bir görüşme ayarlayabiliriz.
 Saygılarımla,
@@ -6381,7 +6381,7 @@
       </c>
       <c r="R64" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -6393,12 +6393,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Miracle Cash&amp;More</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -6409,7 +6409,7 @@
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -6449,18 +6449,18 @@
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>Merhaba Zeynep, İngilizce konuşma pratiği ve gelişim takibi konusunda Konuşarak Öğren ile çalışan ekiplerin, global toplantılarda kendilerini daha güvende hissettiğini görüyoruz. İlgini çekerse, detayları paylaşmak isterim.</t>
+          <t>Merhaba Zeynep Hanım, İngilizce konuşma pratiği ve gelişim takibi konusunda Konuşarak Öğren ile çalışan ekiplerin, global toplantılarda kendilerini daha güvende hissettiğini görüyoruz. İlgini çekerse, detayları paylaşmak isterim.</t>
         </is>
       </c>
       <c r="P65" t="inlineStr">
         <is>
           <t>Konu: Çalışanlarınızın İngilizce Konuşma Yetkinliğini Artırın
-Merhaba Zeynep,
+Merhaba Zeynep Hanım,
 Şirketinizdeki çalışanların global toplantılarda daha fazla özgüvenle konuşmalarını sağlamak için Konuşarak Öğren olarak online İngilizce konuşma pratiği ve gelişim takibi sunuyoruz. Ekibinizin iletişim becerilerini geliştirmesi, uluslararası etkileşimlerde daha etkili olmalarına katkı sağlayacaktır. 
 Detayları paylaşmak için bir görüşme ayarlamak ister misin?
 İyi çalışmalar,
@@ -6474,7 +6474,7 @@
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -6547,13 +6547,13 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>Merhaba Emre, global toplantılarda İngilizce iletişim zorluklarının farkındayım. Konuşarak Öğren, ekip üyelerinizin konuşma özgüvenini artırarak bu süreci kolaylaştırabilir. Detayları paylaşmak isterim!</t>
+          <t>Merhaba Emre Bey, global toplantılarda İngilizce iletişim zorluklarının farkındayım. Konuşarak Öğren, ekip üyelerinizin konuşma özgüvenini artırarak bu süreci kolaylaştırabilir. Detayları paylaşmak isterim!</t>
         </is>
       </c>
       <c r="P66" t="inlineStr">
         <is>
           <t>Konu: İngilizce İletişimde Güçlenin
-Merhaba Emre,
+Merhaba Emre Bey,
 Ekiplerinizin global toplantılarda etkili iletişim kurabilmesi için İngilizce konuşma pratiğine ihtiyaç duyduğunu düşünüyorum. Konuşarak Öğren, çalışanlarınızın konuşma özgüvenini artırarak bu zorlukları aşmalarına yardımcı olabilir. Online platformumuz sayesinde gelişim takibi ve raporlama da sağlıyoruz. 
 Detayları görüşmek ister misiniz?
 İyi çalışmalar,
@@ -6640,7 +6640,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>Merhaba Enes, İngilizce konuşma pratiği üzerine sunduğumuz çözümlerle çalışanların kendine güvenini artırarak global iletişimini güçlendirmeyi hedefliyoruz. Bu konuda daha fazla bilgi almak isterseniz, görüşmek isterim.</t>
+          <t>Merhaba Enes Bey, İngilizce konuşma pratiği üzerine sunduğumuz çözümlerle çalışanların kendine güvenini artırarak global iletişimini güçlendirmeyi hedefliyoruz. Bu konuda daha fazla bilgi almak isterseniz, görüşmek isterim.</t>
         </is>
       </c>
       <c r="P67" t="inlineStr">
@@ -6674,12 +6674,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Nevita</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -6690,7 +6690,7 @@
       <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -6730,18 +6730,18 @@
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>95</t>
         </is>
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>Merhaba Sadullah, İngilizce konuşma pratiği ile çalışanlarınızın global toplantılara hazırlığını artırabileceğinizi biliyor muydunuz? Konuşarak Öğren olarak bu konuda destek sunabiliriz. Detaylı bilgi için bağlantı kuralım!</t>
+          <t>Merhaba Sadullah Bey, İngilizce konuşma pratiği ile çalışanlarınızın global toplantılara hazırlığını artırabileceğinizi biliyor muydunuz? Konuşarak Öğren olarak bu konuda destek sunabiliriz. Detaylı bilgi için bağlantı kuralım!</t>
         </is>
       </c>
       <c r="P68" t="inlineStr">
         <is>
           <t>Konu: Çalışanlarınızın İngilizce Konuşma Becerilerini Geliştirin
-Merhaba Sadullah,
+Merhaba Sadullah Bey,
 Kurumsal ekibinizin İngilizce konuşma becerilerini geliştirmek ve global toplantılara daha iyi hazırlanmaları için etkili bir çözüm arıyorsanız, Konuşarak Öğren size yardımcı olabilir. Online platformumuz, çalışanlarınıza özgü gelişim takibi ve raporlama imkanı sunarak, kendilerine olan güvenlerini artırmalarını sağlıyor.
 Daha fazla bilgi almak isterseniz, size uygun bir zaman diliminde görüşmeyi çok isterim.
 İyi çalışmalar,
@@ -6755,7 +6755,7 @@
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -6767,12 +6767,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Eyüpsultan Belediyesi</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>Genel Müdür Yardımcısı (İnsan Kaynakları)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -6783,7 +6783,7 @@
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -6823,12 +6823,12 @@
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>95</t>
         </is>
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>Merhaba İkbal Hanım, çalışanlarınızın İngilizce konuşma becerilerini geliştirmek, global toplantılara hazır olmalarını sağlamak için online pratik imkanı sunuyoruz. Ekibinizin iletişim becerilerini artırmak için nasıl bir destek sağlayabileceğimizi konuşmak ister misiniz?</t>
+          <t>Merhaba Ikbal Bey, çalışanlarınızın İngilizce konuşma becerilerini geliştirmek, global toplantılara hazır olmalarını sağlamak için online pratik imkanı sunuyoruz. Ekibinizin iletişim becerilerini artırmak için nasıl bir destek sağlayabileceğimizi konuşmak ister misiniz?</t>
         </is>
       </c>
       <c r="P69" t="inlineStr">
@@ -6848,7 +6848,7 @@
       </c>
       <c r="R69" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -6921,13 +6921,13 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>Merhaba Ahmet, global toplantılarda etkili iletişim ve ekip üyelerinin konuşma özgüvenini artırma ihtiyacınızı anlıyorum. Konuşarak Öğren ile İngilizce pratik yaparak bu hedeflere ulaşmanıza yardımcı olabiliriz. Görüşmek ister misiniz?</t>
+          <t>Merhaba Ahmet Bey, global toplantılarda etkili iletişim ve ekip üyelerinin konuşma özgüvenini artırma ihtiyacınızı anlıyorum. Konuşarak Öğren ile İngilizce pratik yaparak bu hedeflere ulaşmanıza yardımcı olabiliriz. Görüşmek ister misiniz?</t>
         </is>
       </c>
       <c r="P70" t="inlineStr">
         <is>
           <t>Konu: Ekip İletişimini Güçlendirin
-Merhaba Ahmet,
+Merhaba Ahmet Bey,
 Şirketinizdeki ekiplerin global toplantılarda etkili iletişim kurabilmesi ve bireylerin konuşma özgüvenini artırabilmesi için online İngilizce pratik imkanı sunuyoruz. Konuşarak Öğren ile çalışanlarınızın İngilizce becerilerini geliştirmesine yardımcı olabiliriz. Bu, HR gelişim hedeflerinize katkıda bulunabilir. İlgilenirseniz, detayları konuşmak isterim.
 Saygılarımla,
 [Adınız]
@@ -7015,13 +7015,13 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>Merhaba Gündem, HR profesyoneli olarak global toplantılardaki iletişim becerilerinin artırılması üzerine konuşmak isterim. Konuşarak Öğren, ekibinizin İngilizce konuşma pratiği yaparak kendine güven kazandırmasına yardımcı olabilir. Görüşmek ister misiniz?</t>
+          <t>Merhaba Gündem Bey, HR profesyoneli olarak global toplantılardaki iletişim becerilerinin artırılması üzerine konuşmak isterim. Konuşarak Öğren, ekibinizin İngilizce konuşma pratiği yaparak kendine güven kazandırmasına yardımcı olabilir. Görüşmek ister misiniz?</t>
         </is>
       </c>
       <c r="P71" t="inlineStr">
         <is>
           <t>Konu: Global Toplantılarda İletişim Becerilerini Geliştirin
-Merhaba Gündem,
+Merhaba Gündem Bey,
 Şirketinizdeki ekiplerin global toplantılarda daha etkili iletişim kurabilmesi için İngilizce konuşma pratiği yapmalarının önemini biliyoruz. Konuşarak Öğren, çalışanlarınızın kendine güven kazanmalarına ve iletişim becerilerini geliştirmelerine yardımcı olabilir. Online platformumuz, gelişim takibi ve raporlama ile destekleniyor. Bu konuyu detaylandırmak için bir görüşme ayarlamak ister misiniz?
 İyi günler dilerim,
 [Adınız]  
@@ -7047,12 +7047,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Tibet / Sultanlar Holding</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Direktörü</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -7063,7 +7063,7 @@
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -7103,18 +7103,18 @@
       </c>
       <c r="N72" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>95</t>
         </is>
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>Merhaba Ersoy, Kurumsal ekiplerin global ortamlarda daha etkili olabilmesi için İngilizce konuşma pratiği yapmalarının önemini biliyorum. Konuşarak Öğren olarak, ekiplerinizin speaking confidence kazanmasına yardımcı olabiliriz. Detayları görüşmek ister misiniz?</t>
+          <t>Merhaba Ersoy Bey, Kurumsal ekiplerin global ortamlarda daha etkili olabilmesi için İngilizce konuşma pratiği yapmalarının önemini biliyorum. Konuşarak Öğren olarak, ekiplerinizin speaking confidence kazanmasına yardımcı olabiliriz. Detayları görüşmek ister misiniz?</t>
         </is>
       </c>
       <c r="P72" t="inlineStr">
         <is>
           <t>Konu: Ekiplerinizin İngilizce Konuşma Yetkinliğini Artırın
-Merhaba Ersoy Polat,
+Merhaba Ersoy Bey Polat,
 Umarım bu mesaj sizi iyi bulur. Şirketinizdeki ekiplerin global toplantılarda daha etkili olabilmesi için İngilizce konuşma pratiği ihtiyaçlarının farkındayım. Konuşarak Öğren olarak, kurumsal ekiplerinize online İngilizce konuşma pratiği sunuyor ve gelişimlerini takip ederek raporlama yapıyoruz. Ekiplerinizin speaking confidence kazanarak uluslararası ortamlarda daha başarılı olmalarına yardımcı olabiliriz. Detayları görüşmek ister misiniz?
 İyi çalışmalar,
 [Adınız]</t>
@@ -7127,7 +7127,7 @@
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -7139,12 +7139,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Platform Gayrimenkul Değerleme ve Danışmanlık A.Ş.</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -7155,7 +7155,7 @@
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -7195,18 +7195,18 @@
       </c>
       <c r="N73" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>85</t>
         </is>
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>Merhaba Berrin, global iş ortamında ekiplerin İngilizce konuşma becerilerini geliştirmeye yönelik bir çözüm sunuyoruz. Çalışanlarınızın güvenle global toplantılara katılmalarına yardımcı olabiliriz. Görüşmek ister misiniz?</t>
+          <t>Merhaba Berrin Bey, global iş ortamında ekiplerin İngilizce konuşma becerilerini geliştirmeye yönelik bir çözüm sunuyoruz. Çalışanlarınızın güvenle global toplantılara katılmalarına yardımcı olabiliriz. Görüşmek ister misiniz?</t>
         </is>
       </c>
       <c r="P73" t="inlineStr">
         <is>
           <t>Konu: Ekiplerinizin İngilizce Yetkinliğini Artırmak
-Merhaba Berrin,
+Merhaba Berrin Bey,
 Gelişen global iş ortamında ekiplerinizin İngilizce konuşma becerilerini artırmak, başarı için kritik bir adım. Konuşarak Öğren olarak, kurumsal ekiplerinize online İngilizce konuşma pratiği sunuyoruz. Bu sayede çalışanlarınızın global toplantılara daha iyi hazırlanmalarını ve kendilerine olan güvenlerini artırmalarını sağlıyoruz. 
 Ekiplerinizin iletişim becerilerini güçlendirmek için bir görüşme ayarlamak ister misiniz?
 Saygılarımla,
@@ -7221,7 +7221,7 @@
       </c>
       <c r="R73" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -7294,13 +7294,13 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>Merhaba Efe, İngilizce konuşma pratiğiyle çalışanlarınızın özgüvenini artırmak ve global toplantılara daha iyi hazırlanmalarını sağlamak için Konuşarak Öğren'in sunduğu çözümleri keşfetmek ister misiniz? Detayları paylaşmak için sabırsızlanıyorum!</t>
+          <t>Merhaba Efe Bey, İngilizce konuşma pratiğiyle çalışanlarınızın özgüvenini artırmak ve global toplantılara daha iyi hazırlanmalarını sağlamak için Konuşarak Öğren'in sunduğu çözümleri keşfetmek ister misiniz? Detayları paylaşmak için sabırsızlanıyorum!</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
         <is>
           <t>Konu: Çalışanlarınızın İletişim Becerelerini Geliştirin
-Merhaba Efe,
+Merhaba Efe Bey,
 Kurumsal ekibinizin global toplantılarda daha etkili olmasını sağlamak için, Konuşarak Öğren olarak online İngilizce konuşma pratiği, gelişim takibi ve raporlama sunuyoruz. Çalışanlarınızın konuşma özgüvenini artırarak, uluslararası ortamlarda daha başarılı olmalarına yardımcı olabiliriz. Bu konuda daha fazla bilgi almak isterseniz, sizinle görüşmeyi çok isterim.
 İyi çalışmalar,
 [İsminiz]</t>
@@ -7386,13 +7386,13 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>Merhaba Sevda, HR süreçlerinde etkili iletişimin önemini biliyorum. Kurumsal ekibinizin İngilizce konuşma pratiği ile gelişim takibi ihtiyacını karşılayabiliriz. Detayları konuşmak ister misiniz?</t>
+          <t>Merhaba Sevda Hanım, HR süreçlerinde etkili iletişimin önemini biliyorum. Kurumsal ekibinizin İngilizce konuşma pratiği ile gelişim takibi ihtiyacını karşılayabiliriz. Detayları konuşmak ister misiniz?</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
           <t>Konu: İletişimde Fark Yaratın
-Merhaba Sevda,
+Merhaba Sevda Hanım,
 HR alanında etkili iletişimin, çalışan gelişimi ve iş süreçlerinde ne kadar kritik olduğunu biliyoruz. Kurumsal ekibinizin İngilizce konuşma pratiği yaparak, global ortamlarda daha etkili olmasını sağlamak için 'Konuşarak Öğren' olarak yanınızdayız. İhtiyaç duydukları anlarda kendilerini ifade edebilmeleri ve toplantılara daha hazır olmaları için destek sunuyoruz. 
 İlgilenirseniz, detayları paylaşmak isterim.
 İyi çalışmalar,
@@ -7479,13 +7479,13 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>Merhaba Hilal, İngilizce konuşma pratiği ile çalışanlarınızın iletişim becerilerini geliştirmelerine yardımcı olabileceğimizi düşünüyorum. Kurumsal ekipler için sunduğumuz çözümleri konuşmak ister misiniz?</t>
+          <t>Merhaba Hilal Hanım, İngilizce konuşma pratiği ile çalışanlarınızın iletişim becerilerini geliştirmelerine yardımcı olabileceğimizi düşünüyorum. Kurumsal ekipler için sunduğumuz çözümleri konuşmak ister misiniz?</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
           <t>Konu: Çalışanlarınızın İngilizce İletişim Becerilerini Geliştirin
-Merhaba Hilal,
+Merhaba Hilal Hanım,
 Şirketinizdeki çalışanların iletişim becerilerini güçlendirmek, global toplantılara daha hazır hale gelmelerini sağlamak için online İngilizce konuşma pratiği sunuyoruz. Hedefe yönelik uygulamalarımızla çalışanların kendilerine olan güvenlerini artırabiliriz. Gelişim takibi ve raporlama ile de süreci daha verimli hale getirebiliriz. Detayları konuşmak isterseniz, size uygun bir zamanda görüşmeyi çok isterim.
 İyi çalışmalar dilerim,
 [Adınız] 
@@ -7512,12 +7512,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>GEMAK GENEL SOGUTMA A.Ş.</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -7528,7 +7528,7 @@
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Tuzla, Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -7568,12 +7568,12 @@
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>85</t>
         </is>
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>Merhaba Ahmet, global toplantılardaki iletişim engellerini aşmak adına çalışanlarınızın İngilizce konuşma pratiğine ihtiyaç duyabileceğini düşünüyorum. Konuşarak Öğren ile bu süreci kolaylaştırabiliriz. Biraz sohbet edelim mi?</t>
+          <t>Merhaba Ahmet Bey, global toplantılardaki iletişim engellerini aşmak adına çalışanlarınızın İngilizce konuşma pratiğine ihtiyaç duyabileceğini düşünüyorum. Konuşarak Öğren ile bu süreci kolaylaştırabiliriz. Biraz sohbet edelim mi?</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
@@ -7595,7 +7595,7 @@
       </c>
       <c r="R77" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -7607,12 +7607,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>EKO TEKSTİL</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -7623,7 +7623,7 @@
       <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -7663,18 +7663,18 @@
       </c>
       <c r="N78" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>95</t>
         </is>
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>Merhaba Fatih, HR alanındaki deneyiminizle, ekiplerin İngilizce iletişim becerilerini geliştirmek için nasıl çözümler aradığınızı merak ediyorum. Konuşarak Öğren ile, çalışanlarınızın global toplantılara daha hazır hale gelmesine yardımcı olabiliriz. Görüşmek ister misiniz?</t>
+          <t>Merhaba Fatih Bey, HR alanındaki deneyiminizle, ekiplerin İngilizce iletişim becerilerini geliştirmek için nasıl çözümler aradığınızı merak ediyorum. Konuşarak Öğren ile, çalışanlarınızın global toplantılara daha hazır hale gelmesine yardımcı olabiliriz. Görüşmek ister misiniz?</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
         <is>
           <t>Konu: Çalışanlarınızın İngilizce İletişim Becerilerini Geliştirin
-Merhaba Fatih,
+Merhaba Fatih Bey,
 HR alanındaki tecrübelerinizle, çalışanlarınızın İngilizce iletişim becerilerini geliştirme ihtiyacını anlıyorum. Konuşarak Öğren olarak, ekibinize online İngilizce konuşma pratiği sunuyoruz. Bu sayede, global toplantılara daha özgüvenli katılmalarını sağlıyor ve gelişimlerini raporluyoruz. Çözümümüz hakkında daha fazla bilgi almak isterseniz, bir görüşme ayarlayalım.
 İyi çalışmalar,
 [İsminiz]</t>
@@ -7687,7 +7687,7 @@
       </c>
       <c r="R78" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -7760,13 +7760,13 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>Merhaba Birgul Hanım, gelişen iş dünyasında çalışanlarınızın İngilizce konuşma becerilerini artırmalarına yardımcı olabileceğimize inanıyorum. Online konuşma pratiği ile ekibinizin global toplantılara daha hazır hale gelmesini sağlayabiliriz. Detayları konuşmak ister misiniz?</t>
+          <t>Merhaba Birgul Bey, gelişen iş dünyasında çalışanlarınızın İngilizce konuşma becerilerini artırmalarına yardımcı olabileceğimize inanıyorum. Online konuşma pratiği ile ekibinizin global toplantılara daha hazır hale gelmesini sağlayabiliriz. Detayları konuşmak ister misiniz?</t>
         </is>
       </c>
       <c r="P79" t="inlineStr">
         <is>
           <t>Konu: Ekiplerinizin İngilizce Konuşma Becerilerini Geliştirin
-Merhaba Birgul Hanım,
+Merhaba Birgul Bey,
 Gelişen iş dünyasında, ekiplerinizin İngilizce konuşma becerilerini geliştirmekte zorluklar yaşadığını biliyorum. Konuşarak Öğren olarak, online İngilizce konuşma pratiği sunarak çalışanlarınızın kendine güvenlerini artırmalarına ve global toplantılara daha iyi hazırlanmalarına yardımcı olabiliriz.
 Görüşmek için uygun bir zaman ayarlamak ister misiniz?
 Saygılarımla,
@@ -7793,12 +7793,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>QTerminals Antalya</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -7809,7 +7809,7 @@
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Antalya, Turkey</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -7849,12 +7849,12 @@
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>90</t>
         </is>
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>Merhaba Emine, çalışanların İngilizce iletişim becerilerini geliştirmek ve bu süreçteki ilerlemeyi takip etmek adına sizlerle tanışmak istedim. Online konuşma pratiği ile ekiplerinizi daha etkili hale getirebiliriz. Görüşmek ister misiniz?</t>
+          <t>Merhaba Emine Hanım, çalışanların İngilizce iletişim becerilerini geliştirmek ve bu süreçteki ilerlemeyi takip etmek adına sizlerle tanışmak istedim. Online konuşma pratiği ile ekiplerinizi daha etkili hale getirebiliriz. Görüşmek ister misiniz?</t>
         </is>
       </c>
       <c r="P80" t="inlineStr">
@@ -7875,7 +7875,7 @@
       </c>
       <c r="R80" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -7887,12 +7887,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Sirena Marine</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları ve İSG Müdürü</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -7903,7 +7903,7 @@
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Bursa, Turkey</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -7943,18 +7943,18 @@
       </c>
       <c r="N81" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>95</t>
         </is>
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>Merhaba Tuğba, kurumsal ekiplerin İngilizce iletişim becerilerini geliştirmelerine yardımcı olmanın önemini biliyorum. Konuşarak Öğren ile online konuşma pratiği sunarak, ekibinizin özgüvenini ve toplantılardaki etkinliğini artırabilirsiniz. Detayları paylaşmak ister misiniz? Sevgiler!</t>
+          <t>Merhaba Tuğba Hanım, kurumsal ekiplerin İngilizce iletişim becerilerini geliştirmelerine yardımcı olmanın önemini biliyorum. Konuşarak Öğren ile online konuşma pratiği sunarak, ekibinizin özgüvenini ve toplantılardaki etkinliğini artırabilirsiniz. Detayları paylaşmak ister misiniz? Sevgiler!</t>
         </is>
       </c>
       <c r="P81" t="inlineStr">
         <is>
           <t>Konu: Ekibinizin İngilizce İletişim Becerilerini Güçlendirin
-Merhaba Tuğba,
+Merhaba Tuğba Hanım,
 Türkiye'deki HR profesyonelleri olarak, kurumsal ekiplerde etkili iletişimin önemini biliyoruz. Konuşarak Öğren olarak, çalışanlarınıza online İngilizce konuşma pratiği sunarak, iletişim becerilerini geliştirmelerine yardımcı olabiliriz. Bu, global toplantılarda daha etkili olmalarını sağlayacak ve özgüvenlerini artıracaktır.
 Daha fazla bilgi almak isterseniz, sizinle görüşmek isterim.
 Sevgiler,
@@ -7970,7 +7970,7 @@
       </c>
       <c r="R81" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -8043,7 +8043,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>Merhaba Latif, HR teknolojileri alanındaki çalışmalarınızı takip ediyorum. Ekibinizin İngilizce konuşma becerilerini geliştirmesi, global toplantılarda daha etkili olmalarını sağlayabilir. Konuşarak Öğren, bu konuda destek olabilir. Detayları paylaşmak isterim.</t>
+          <t>Merhaba Latif Bey, HR teknolojileri alanındaki çalışmalarınızı takip ediyorum. Ekibinizin İngilizce konuşma becerilerini geliştirmesi, global toplantılarda daha etkili olmalarını sağlayabilir. Konuşarak Öğren, bu konuda destek olabilir. Detayları paylaşmak isterim.</t>
         </is>
       </c>
       <c r="P82" t="inlineStr">
@@ -8136,13 +8136,13 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>Merhaba Lara, HR alanındaki deneyiminizle, çalışanların İngilizce konuşma becerilerini geliştirmesi için etkili çözümler sunabileceğimize inanıyorum. Konuşarak Öğren ile ekibinizin iletişim yeteneklerini güçlendirebiliriz. Detayları paylaşmak ister misiniz?</t>
+          <t>Merhaba Lara Hanım, HR alanındaki deneyiminizle, çalışanların İngilizce konuşma becerilerini geliştirmesi için etkili çözümler sunabileceğimize inanıyorum. Konuşarak Öğren ile ekibinizin iletişim yeteneklerini güçlendirebiliriz. Detayları paylaşmak ister misiniz?</t>
         </is>
       </c>
       <c r="P83" t="inlineStr">
         <is>
           <t>Konu: Çalışanlarınızın İngilizce Konuşma Becerilerini Geliştirin
-Merhaba Lara,
+Merhaba Lara Hanım,
 Kurumsal ekibinizin global toplantılara daha iyi hazırlanabilmesi için İngilizce konuşma becerilerini geliştirmek önemli bir konu. Konuşarak Öğren olarak, online İngilizce konuşma pratiği ile çalışanlarınızın güvenini artırmayı ve gelişimlerini düzenli olarak takip etmeyi sağlıyoruz. Bu konuda sizinle bir görüşme yapmak isterim. 
 İyi çalışmalar dilerim,
 [İsminiz]  
@@ -8229,13 +8229,13 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>Merhaba Gülşah, global iş ortamında ekiplerin İngilizce iletişim becerilerini artırma konusundaki çabalarınızı duydum. Kurumsal ekipler için online İngilizce pratik imkanı sunarak bu hedefe ulaşmalarına yardımcı olabiliriz. Detayları paylaşmak isterim.</t>
+          <t>Merhaba Gülşah Hanım, global iş ortamında ekiplerin İngilizce iletişim becerilerini artırma konusundaki çabalarınızı duydum. Kurumsal ekipler için online İngilizce pratik imkanı sunarak bu hedefe ulaşmalarına yardımcı olabiliriz. Detayları paylaşmak isterim.</t>
         </is>
       </c>
       <c r="P84" t="inlineStr">
         <is>
           <t>Konu: Ekiplerin İngilizce İletişim Becerilerini Geliştirin
-Merhaba Gülşah,
+Merhaba Gülşah Hanım,
 Global iş ortamında ekiplerinizin İngilizce iletişim becerilerini artırmak için etkili bir yol arıyorsanız, size yardımcı olabiliriz. Konuşarak Öğren olarak, kurumsal ekipler için online İngilizce konuşma pratiği sunuyoruz. Ekiplerinizin uluslararası toplantılara daha iyi hazırlanması ve kendine güven eksikliklerini gidermesi için birlikte çalışabiliriz. 
 Detayları paylaşmak isterim.
 Saygılarımla,
@@ -8322,13 +8322,13 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>Merhaba Yasemin, HR alanındaki deneyiminizle, ekiplerin İngilizce iletişim becerilerini geliştirmesine yardımcı olma konusunda katkınızın büyük olduğunu düşünüyorum. Konuşarak Öğren ile ekiplerinizi global toplantılara daha iyi hazırlayabilirsiniz. Daha fazla bilgi için bağlantı kuralım!</t>
+          <t>Merhaba Yasemin Hanım, HR alanındaki deneyiminizle, ekiplerin İngilizce iletişim becerilerini geliştirmesine yardımcı olma konusunda katkınızın büyük olduğunu düşünüyorum. Konuşarak Öğren ile ekiplerinizi global toplantılara daha iyi hazırlayabilirsiniz. Daha fazla bilgi için bağlantı kuralım!</t>
         </is>
       </c>
       <c r="P85" t="inlineStr">
         <is>
           <t>Konu: Ekip İletişimini Güçlendirin
-Merhaba Yasemin,
+Merhaba Yasemin Hanım,
 Kurumsal ekiplerin İngilizce iletişim becerilerini geliştirmeleri, global toplantılarda etkinliklerini artırmak için kritik. Konuşarak Öğren, ekiplerinize çevrimiçi İngilizce konuşma pratiği sunarak bu süreci destekliyor. Gelişim takibi ve raporlama ile ilerlemenizi kolayca takip edebilirsiniz. 
 Detayları konuşmak için bir görüşme ayarlamak ister misiniz?
 Saygılarımla,
@@ -8416,13 +8416,13 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>Merhaba Onur, şirketinizdeki ekiplerin İngilizce konuşma pratiği ihtiyacını gözlemledim. Konuşarak Öğren ile speaking confidence ve global toplantılara hazırlık süreçlerinizi güçlendirebiliriz. Detayları paylaşmak ister misiniz?</t>
+          <t>Merhaba Onur Bey, şirketinizdeki ekiplerin İngilizce konuşma pratiği ihtiyacını gözlemledim. Konuşarak Öğren ile speaking confidence ve global toplantılara hazırlık süreçlerinizi güçlendirebiliriz. Detayları paylaşmak ister misiniz?</t>
         </is>
       </c>
       <c r="P86" t="inlineStr">
         <is>
           <t>Konu: Ekiplerinizin İngilizce İletişim Becerilerini Geliştirin
-Merhaba Onur,
+Merhaba Onur Bey,
 Gelişmiş iletişim becerileri, global toplantılarda etkin olmanın anahtarı. Konuşarak Öğren olarak, kurumsal ekiplerinize özel online İngilizce konuşma pratiği sunuyoruz. Ekip üyelerinizin speaking confidence ve global meeting readiness düzeylerini artırarak, uluslararası arenada daha etkili olmalarını sağlamak istiyoruz. 
 Detayları görüşmek için uygun bir zamanınız var mı?
 İyi çalışmalar,
@@ -8449,12 +8449,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Auto Life Center</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -8465,7 +8465,7 @@
       <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -8505,18 +8505,18 @@
       </c>
       <c r="N87" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>90</t>
         </is>
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>Merhaba Duygu, HR alanındaki tecrübelerinizle ekibinizin global toplantılarda daha özgüvenli olmasına katkı sağlamak için online İngilizce konuşma pratiği sunuyoruz. Bu konuda daha fazla bilgi almak ister misiniz?</t>
+          <t>Merhaba Duygu Hanım, HR alanındaki tecrübelerinizle ekibinizin global toplantılarda daha özgüvenli olmasına katkı sağlamak için online İngilizce konuşma pratiği sunuyoruz. Bu konuda daha fazla bilgi almak ister misiniz?</t>
         </is>
       </c>
       <c r="P87" t="inlineStr">
         <is>
           <t>Konu: Ekibinizin İngilizce Konuşma Becerilerini Geliştirin
-Merhaba Duygu,
+Merhaba Duygu Hanım,
 Şirketinizin global toplantılarda daha etkin bir şekilde yer alabilmesi için, ekibinize özel online İngilizce konuşma pratiği sunuyoruz. Bu program, çalışanlarınızın kendilerine olan güvenini artırarak, uluslararası işbirliklerinde daha başarılı olmalarına yardımcı olabilir. 
 Detayları konuşmak isterseniz, size yardımcı olmaktan mutluluk duyarım.
 İyi çalışmalar,
@@ -8531,7 +8531,7 @@
       </c>
       <c r="R87" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -8543,12 +8543,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>PozitifTech</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -8559,7 +8559,7 @@
       <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -8599,18 +8599,18 @@
       </c>
       <c r="N88" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>Merhaba Nejla, global iş ortamında İngilizce konuşma becerilerinin önemini biliyorum. Kurumsal ekipler için sunduğumuz online konuşma pratiği ile iletişim becerilerini geliştirmek konusunda yardımcı olabilirim. Görüşmek ister misiniz?</t>
+          <t>Merhaba Nejla Hanım, global iş ortamında İngilizce konuşma becerilerinin önemini biliyorum. Kurumsal ekipler için sunduğumuz online konuşma pratiği ile iletişim becerilerini geliştirmek konusunda yardımcı olabilirim. Görüşmek ister misiniz?</t>
         </is>
       </c>
       <c r="P88" t="inlineStr">
         <is>
           <t>Konu: Takımınızın İngilizce Konuşma Becerilerini Geliştirin
-Merhaba Nejla,
+Merhaba Nejla Hanım,
 Gelişen global iş ortamında, çalışanların İngilizce konuşma yeteneklerinin yetersizliği büyük bir zorluk oluşturuyor. Konuşarak Öğren olarak, ekiplerinizi online İngilizce konuşma pratiği ile destekleyerek, iletişim becerilerini artırmayı ve global toplantılarda daha etkili olmalarını sağlamayı hedefliyoruz.
 Bu süreçte, gelişim takibi ve raporlama ile sürekli ilerleme kaydetmelerine yardımcı oluyoruz. Şirketinizin bu konuda nasıl bir destek alabileceğini konuşmak ister misiniz?
 İyi çalışmalar,
@@ -8624,7 +8624,7 @@
       </c>
       <c r="R88" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -8636,12 +8636,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>MAY Tohum</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -8652,7 +8652,7 @@
       <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Bursa, Turkey</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -8692,18 +8692,18 @@
       </c>
       <c r="N89" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>95</t>
         </is>
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>Merhaba Sebla, global iş ortamında ekiplerin İngilizce iletişim becerilerini artırmak adına nasıl bir yol izlediğinizi merak ediyorum. Konuşarak Öğren ile kurumsal ekiplere yönelik çözümler sunuyoruz. İlgilenirseniz, detayları konuşalım.</t>
+          <t>Merhaba Sebla Hanım, global iş ortamında ekiplerin İngilizce iletişim becerilerini artırmak adına nasıl bir yol izlediğinizi merak ediyorum. Konuşarak Öğren ile kurumsal ekiplere yönelik çözümler sunuyoruz. İlgilenirseniz, detayları konuşalım.</t>
         </is>
       </c>
       <c r="P89" t="inlineStr">
         <is>
           <t>Konu: Ekiplerinizin İngilizce İletişim Becerilerini Güçlendirin
-Merhaba Sebla,
+Merhaba Sebla Hanım,
 Gelişen global iş ortamında, ekiplerin İngilizce konuşma pratiği yaparak kendilerine güven kazanması ve uluslararası toplantılara hazır hale gelmesi oldukça önemli. Konuşarak Öğren olarak, kurumsal ekipler için online İngilizce konuşma pratiği sunuyoruz. Çalışanlarınızın iletişim becerilerini geliştirmeye yönelik çözümlerimizle, gelişim takibi ve raporlama süreçlerini de destekliyoruz. 
 Detayları konuşmak isterseniz, memnuniyetle yardımcı olurum.
 İyi çalışmalar,
@@ -8717,7 +8717,7 @@
       </c>
       <c r="R89" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -8790,13 +8790,13 @@
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>Merhaba Nurdan, İngilizce konuşma pratiği eksikliğinin ekiplerinizdeki global toplantılara hazırlığı etkilediğini biliyoruz. Konuşarak Öğren ile bu süreci geliştirmek ve ekiplerinizin özgüvenini artırmak hakkında konuşmak ister misiniz?</t>
+          <t>Merhaba Nurdan Bey, İngilizce konuşma pratiği eksikliğinin ekiplerinizdeki global toplantılara hazırlığı etkilediğini biliyoruz. Konuşarak Öğren ile bu süreci geliştirmek ve ekiplerinizin özgüvenini artırmak hakkında konuşmak ister misiniz?</t>
         </is>
       </c>
       <c r="P90" t="inlineStr">
         <is>
           <t>Konu: Ekipleriniz için İngilizce Konuşma Pratiği
-Merhaba Nurdan,
+Merhaba Nurdan Bey,
 Umarım iyisinizdir! Şirketinizdeki ekiplerin global toplantılara daha etkili katılım göstermesi için İngilizce konuşma pratiğinin önemini biliyorum. Konuşarak Öğren olarak, online platformumuz ile ekip üyelerinizin speaking confidence ve global meeting readiness becerilerini geliştirmelerine yardımcı olabiliriz. 
 Sizinle bu konuda daha detaylı konuşmak isterim. Uygun olduğunuzda bir görüşme ayarlayabilir miyiz?
 İyi çalışmalar,
@@ -8822,12 +8822,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>Healmedy</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -8838,7 +8838,7 @@
       <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -8878,12 +8878,12 @@
       </c>
       <c r="N91" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>95</t>
         </is>
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>Merhaba Banu, İngilizce konuşma pratiği ile çalışanların global toplantılara daha hazır hale gelmesini sağlıyoruz. Ekibinizin iletişim becerilerini güçlendirmek, uluslararası iletişimdeki özgüvenlerini artırmak için yardımcı olabiliriz. Görüşelim mi?</t>
+          <t>Merhaba Banu Hanım, İngilizce konuşma pratiği ile çalışanların global toplantılara daha hazır hale gelmesini sağlıyoruz. Ekibinizin iletişim becerilerini güçlendirmek, uluslararası iletişimdeki özgüvenlerini artırmak için yardımcı olabiliriz. Görüşelim mi?</t>
         </is>
       </c>
       <c r="P91" t="inlineStr">
@@ -8902,7 +8902,7 @@
       </c>
       <c r="R91" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -8914,12 +8914,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>FUPS BANK</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Müdürü</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -8930,7 +8930,7 @@
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>Istanbul, Turkey</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -8970,7 +8970,7 @@
       </c>
       <c r="N92" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>95</t>
         </is>
       </c>
       <c r="O92" t="inlineStr">
@@ -8995,7 +8995,7 @@
       </c>
       <c r="R92" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -9068,7 +9068,7 @@
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>Merhaba Leyla, İngilizce konuşma pratiği ile çalışanların kendine güvenini artırmanın ve uluslararası toplantılara hazırlanmanın ne kadar önemli olduğunu biliyorum. Konuşarak Öğren olarak bu alanda destek olabileceğimizi düşünüyorum. Bağlantıda kalalım!</t>
+          <t>Merhaba Leyla Hanım, İngilizce konuşma pratiği ile çalışanların kendine güvenini artırmanın ve uluslararası toplantılara hazırlanmanın ne kadar önemli olduğunu biliyorum. Konuşarak Öğren olarak bu alanda destek olabileceğimizi düşünüyorum. Bağlantıda kalalım!</t>
         </is>
       </c>
       <c r="P93" t="inlineStr">
@@ -9161,13 +9161,13 @@
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>Merhaba Ferda, HR profesyonellerinin İngilizce iletişim becerilerini güçlendirmek için online konuşma pratiği sunuyoruz. Takımınızın global işbirliğinde daha hazır hale gelmesine yardımcı olabiliriz. Görüşmek ister misiniz?</t>
+          <t>Merhaba Ferda Hanım, HR profesyonellerinin İngilizce iletişim becerilerini güçlendirmek için online konuşma pratiği sunuyoruz. Takımınızın global işbirliğinde daha hazır hale gelmesine yardımcı olabiliriz. Görüşmek ister misiniz?</t>
         </is>
       </c>
       <c r="P94" t="inlineStr">
         <is>
           <t>Konu: Takımınız için İngilizce Konuşma Pratiği 
-Merhaba Ferda, 
+Merhaba Ferda Hanım, 
 Şirketinizin HR ekibinin global işbirliğini güçlendirmek için etkili bir çözüm arayışında olduğunu biliyorum. Konuşarak Öğren olarak, online İngilizce konuşma pratiği sunarak çalışanlarınızın iletişim becerilerini geliştirmelerine yardımcı olabiliriz. Bu sayede, global toplantılara daha hazır bir şekilde katılabilirler. Gelişim takibi ve raporlama ile süreci daha da verimli hale getiriyoruz. 
 İlgilenirseniz, detayları konuşmak için bir görüşme ayarlayabiliriz.
 İyi çalışmalar, 
@@ -9254,13 +9254,13 @@
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>Merhaba Müzeyyen, iletişim becerilerini geliştirmek için harika bir fırsat sunuyoruz! Kurumsal ekipler için İngilizce konuşma pratiği ve gelişim raporlaması ile global iletişimi güçlendirmek istemez misin? Detayları paylaşmak isterim.</t>
+          <t>Merhaba Müzeyyen Hanım, iletişim becerilerini geliştirmek için harika bir fırsat sunuyoruz! Kurumsal ekipler için İngilizce konuşma pratiği ve gelişim raporlaması ile global iletişimi güçlendirmek istemez misin? Detayları paylaşmak isterim.</t>
         </is>
       </c>
       <c r="P95" t="inlineStr">
         <is>
           <t>Konu: Kurumsal Ekipler İçin İngilizce Konuşma Pratiği
-Merhaba Müzeyyen,
+Merhaba Müzeyyen Hanım,
 Çalışanlarınızın İngilizce konuşma becerilerini artırarak global toplantılara daha hazırlıklı olmalarını sağlamak istiyorsanız, 'Konuşarak Öğren' olarak size destek olabiliriz. Online İngilizce konuşma pratiği sunarak, ekibinizin kendine güvenini artırmayı ve gelişimlerini takip etmeyi hedefliyoruz. İlgilenirseniz, detayları paylaşmak isterim.
 Saygılarımla,
 [Adınız]</t>
@@ -9346,13 +9346,13 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>Merhaba Yağmur, İngilizce konuşma pratiği ve global toplantılara hazırlık konusunda ekibinize destek olabileceğimizi düşünüyorum. Konuşarak Öğren ile iletişim becerilerinizi geliştirebilir ve daha etkili bir şekilde global platformlarda yer alabilirsiniz. Detaylar için bir sohbet edelim mi?</t>
+          <t>Merhaba Yağmur Hanım, İngilizce konuşma pratiği ve global toplantılara hazırlık konusunda ekibinize destek olabileceğimizi düşünüyorum. Konuşarak Öğren ile iletişim becerilerinizi geliştirebilir ve daha etkili bir şekilde global platformlarda yer alabilirsiniz. Detaylar için bir sohbet edelim mi?</t>
         </is>
       </c>
       <c r="P96" t="inlineStr">
         <is>
           <t>Konu: Global Toplantılara Daha Hazır Ekipler İçin
-Merhaba Yağmur,
+Merhaba Yağmur Hanım,
 Kurumsal ekibinizin İngilizce konuşma pratiği eksikliği ile başa çıkmak için size yardımcı olabileceğimize inanıyorum. Konuşarak Öğren, ekiplerinize online İngilizce konuşma pratiği, bireysel gelişim takibi ve raporlama sunarak, global toplantılara daha iyi hazırlanmalarına destek oluyor.
 Bu konuda bir görüşme yapmayı ister misiniz? 
 Saygılarımla,
@@ -9440,7 +9440,7 @@
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>Merhaba Betül, HR alanında çalışan biri olarak, çalışanların İngilizce konuşma güvenini artırmak ve global toplantılara hazırlık süreçlerini kolaylaştırmak adına size yardımcı olabileceğimi düşünüyorum. Detayları paylaşmak ister misiniz?</t>
+          <t>Merhaba Betül Hanım, HR alanında çalışan biri olarak, çalışanların İngilizce konuşma güvenini artırmak ve global toplantılara hazırlık süreçlerini kolaylaştırmak adına size yardımcı olabileceğimi düşünüyorum. Detayları paylaşmak ister misiniz?</t>
         </is>
       </c>
       <c r="P97" t="inlineStr">
@@ -9472,12 +9472,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>To be verified from LinkedIn profile/company page</t>
+          <t>CR Canreis Group</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>HR / People Professional - to verify</t>
+          <t>İnsan Kaynakları Direktörü</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -9488,7 +9488,7 @@
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Turkey - to verify</t>
+          <t>İzmir, Turkey</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -9528,12 +9528,12 @@
       </c>
       <c r="N98" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>Merhaba Yeliz, İngilizce konuşma pratiği konusundaki deneyimlerinizi merak ediyorum. Takımınızın global toplantılarda daha etkili olabilmesi için pratik yapma fırsatları sunuyoruz. İlgilenir misiniz?</t>
+          <t>Merhaba Yeliz Hanım, İngilizce konuşma pratiği konusundaki deneyimlerinizi merak ediyorum. Takımınızın global toplantılarda daha etkili olabilmesi için pratik yapma fırsatları sunuyoruz. İlgilenir misiniz?</t>
         </is>
       </c>
       <c r="P98" t="inlineStr">
@@ -9553,7 +9553,7 @@
       </c>
       <c r="R98" t="inlineStr">
         <is>
-          <t>new_enriched_needs_manual_verification</t>
+          <t>verified_message_ready</t>
         </is>
       </c>
     </row>
@@ -9626,13 +9626,13 @@
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>Merhaba Busra, HR profesyoneli olarak ekiplerinizin İngilizce konuşma becerilerini geliştirmesine katkı sağlamak ilginizi çekebilir. Konuşarak Öğren ile online pratik yaparak, çalışanların güvenle iletişim kurmalarını sağlama fırsatını keşfedelim!</t>
+          <t>Merhaba Busra Hanım, HR profesyoneli olarak ekiplerinizin İngilizce konuşma becerilerini geliştirmesine katkı sağlamak ilginizi çekebilir. Konuşarak Öğren ile online pratik yaparak, çalışanların güvenle iletişim kurmalarını sağlama fırsatını keşfedelim!</t>
         </is>
       </c>
       <c r="P99" t="inlineStr">
         <is>
           <t>Konu: Ekiplerinizin İletişim Becerilerini Geliştirin
-Merhaba Busra,
+Merhaba Busra Hanım,
 HR alanındaki deneyiminiz ile çalışanlarınızın İngilizce konuşma pratiği yaparak iletişim becerilerini geliştirmesine katkıda bulunmak isteyebilirsiniz. Konuşarak Öğren, kurumsal ekipler için özel olarak tasarlanmış online pratik programları sunuyor. Bu sayede, çalışanlarınızın konuşma özgüveni artarken, global toplantılara daha iyi hazırlanabilecekler. Daha fazla bilgi almak isterseniz, memnuniyetle görüşürüm.
 İyi günler dilerim,
 [Adınız]</t>
@@ -9718,13 +9718,13 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>Merhaba Mehmet, HR profesyoneli olarak, çalışanlarınızın global toplantılara daha iyi hazırlanmaları için İngilizce konuşma becerilerini geliştirmeleri gerektiğini biliyorum. Konuşarak Öğren, ekibinize online pratik imkanı sunarak bu süreci kolaylaştırabilir. Detayları paylaşmak isterim.</t>
+          <t>Merhaba Mehmet Bey, HR profesyoneli olarak, çalışanlarınızın global toplantılara daha iyi hazırlanmaları için İngilizce konuşma becerilerini geliştirmeleri gerektiğini biliyorum. Konuşarak Öğren, ekibinize online pratik imkanı sunarak bu süreci kolaylaştırabilir. Detayları paylaşmak isterim.</t>
         </is>
       </c>
       <c r="P100" t="inlineStr">
         <is>
           <t>Konu: Çalışanlarınızın İngilizce Konuşma Becerilerini Geliştirin
-Merhaba Mehmet,
+Merhaba Mehmet Bey,
 Şirketinizin global toplantılarda etkili iletişim kurabilmesi için çalışanların İngilizce konuşma becerilerini geliştirmesi kritik. Konuşarak Öğren, kurumsal ekipler için online İngilizce konuşma pratiği, gelişim takibi ve raporlama sunarak bu ihtiyacı karşılıyor.
 Ekibinizin güvenle İngilizce konuşmasını sağlamaya yardımcı olabiliriz. Bir görüşme ayarlayıp detayları konuşmayı çok isterim.
 İyi çalışmalar,
@@ -9813,7 +9813,7 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>Merhaba Duygu, kurumsal ekiplerin İngilizce konuşma pratiği ve gelişim takibi konusunda sağladığımız çözümlerle ilgili konuşmak isterim. Çalışanlarınızın global iletişim becerilerini artırmalarına nasıl destek olabileceğimize bakalım mı?</t>
+          <t>Merhaba Duygu Hanım, kurumsal ekiplerin İngilizce konuşma pratiği ve gelişim takibi konusunda sağladığımız çözümlerle ilgili konuşmak isterim. Çalışanlarınızın global iletişim becerilerini artırmalarına nasıl destek olabileceğimize bakalım mı?</t>
         </is>
       </c>
       <c r="P101" t="inlineStr">

</xml_diff>